<commit_message>
updates to additional_data folder
</commit_message>
<xml_diff>
--- a/additional_data/lookup_tables/ausPH_AusPol_mapping.xlsx
+++ b/additional_data/lookup_tables/ausPH_AusPol_mapping.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindsaykatz/Documents/RA/hansard/data/lookup_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindsaykatz/Documents/RA/hansard/additional_data/lookup_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16890E5D-BFC1-044D-A136-B9809AE82545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6ACC0FC-3076-F248-8BED-4AAB71C9A3A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5560" yWindow="-20580" windowWidth="27640" windowHeight="16360" xr2:uid="{3F854667-67DD-A44E-A8BA-9046689ACB2E}"/>
+    <workbookView xWindow="0" yWindow="840" windowWidth="27640" windowHeight="16360" xr2:uid="{3F854667-67DD-A44E-A8BA-9046689ACB2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$1212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$1213</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7282" uniqueCount="4813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7335" uniqueCount="4844">
   <si>
     <t>uniqueID</t>
   </si>
@@ -14477,6 +14477,99 @@
   </si>
   <si>
     <t>Wolahan, Keith</t>
+  </si>
+  <si>
+    <t>Thorpe</t>
+  </si>
+  <si>
+    <t>Lidia</t>
+  </si>
+  <si>
+    <t>Thorpe1973</t>
+  </si>
+  <si>
+    <t>Lidia Thorpe</t>
+  </si>
+  <si>
+    <t>Coffey, Renee</t>
+  </si>
+  <si>
+    <t>Boele, Nicolette</t>
+  </si>
+  <si>
+    <t>French, Tom</t>
+  </si>
+  <si>
+    <t>Holzberger, Rowan</t>
+  </si>
+  <si>
+    <t>Smith, Matt</t>
+  </si>
+  <si>
+    <t>Abdo, Basem</t>
+  </si>
+  <si>
+    <t>Berry, Carol</t>
+  </si>
+  <si>
+    <t>Penfold, Alison</t>
+  </si>
+  <si>
+    <t>Aldred, Mary</t>
+  </si>
+  <si>
+    <t>Venning, Tom</t>
+  </si>
+  <si>
+    <t>Chaffey, Jamie</t>
+  </si>
+  <si>
+    <t>Rebello, Leon</t>
+  </si>
+  <si>
+    <t>Coffey</t>
+  </si>
+  <si>
+    <t>Boele</t>
+  </si>
+  <si>
+    <t>French</t>
+  </si>
+  <si>
+    <t>Holzberger</t>
+  </si>
+  <si>
+    <t>Abdo</t>
+  </si>
+  <si>
+    <t>Penfold</t>
+  </si>
+  <si>
+    <t>Venning</t>
+  </si>
+  <si>
+    <t>Chaffey</t>
+  </si>
+  <si>
+    <t>Rebello</t>
+  </si>
+  <si>
+    <t>Leon</t>
+  </si>
+  <si>
+    <t>Tom</t>
+  </si>
+  <si>
+    <t>Renee</t>
+  </si>
+  <si>
+    <t>Nicolette</t>
+  </si>
+  <si>
+    <t>Basem</t>
+  </si>
+  <si>
+    <t>Carol</t>
   </si>
 </sst>
 </file>
@@ -14526,7 +14619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -14549,6 +14642,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -14864,7 +14960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19D0AC81-670F-3C42-86B4-43C7337F72FB}">
-  <dimension ref="A1:G1246"/>
+  <dimension ref="A1:G1259"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
@@ -39530,63 +39626,63 @@
         <v>26665</v>
       </c>
     </row>
-    <row r="1116" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1116" s="6" t="s">
-        <v>4347</v>
+    <row r="1116" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1116" s="9" t="s">
+        <v>4815</v>
       </c>
       <c r="B1116" s="2">
-        <v>282212</v>
+        <v>280304</v>
       </c>
       <c r="C1116" s="2" t="s">
-        <v>4348</v>
+        <v>4813</v>
       </c>
       <c r="D1116" s="2" t="s">
-        <v>4349</v>
+        <v>4814</v>
       </c>
       <c r="E1116" s="2" t="s">
-        <v>4350</v>
+        <v>4816</v>
       </c>
       <c r="F1116" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G1116" s="2"/>
+      <c r="G1116" s="3"/>
     </row>
     <row r="1117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1117" s="6" t="s">
-        <v>4351</v>
-      </c>
-      <c r="B1117" s="2" t="s">
-        <v>4352</v>
+        <v>4347</v>
+      </c>
+      <c r="B1117" s="2">
+        <v>282212</v>
       </c>
       <c r="C1117" s="2" t="s">
-        <v>4353</v>
+        <v>4348</v>
       </c>
       <c r="D1117" s="2" t="s">
-        <v>4354</v>
+        <v>4349</v>
       </c>
       <c r="E1117" s="2" t="s">
-        <v>4355</v>
+        <v>4350</v>
       </c>
       <c r="F1117" s="2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="G1117" s="2"/>
     </row>
     <row r="1118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1118" s="6" t="s">
-        <v>4356</v>
+        <v>4351</v>
       </c>
       <c r="B1118" s="2" t="s">
-        <v>4357</v>
+        <v>4352</v>
       </c>
       <c r="C1118" s="2" t="s">
-        <v>4358</v>
+        <v>4353</v>
       </c>
       <c r="D1118" s="2" t="s">
-        <v>205</v>
+        <v>4354</v>
       </c>
       <c r="E1118" s="2" t="s">
-        <v>4359</v>
+        <v>4355</v>
       </c>
       <c r="F1118" s="2" t="s">
         <v>11</v>
@@ -39595,130 +39691,130 @@
     </row>
     <row r="1119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1119" s="6" t="s">
-        <v>4360</v>
+        <v>4356</v>
       </c>
       <c r="B1119" s="2" t="s">
-        <v>4361</v>
+        <v>4357</v>
       </c>
       <c r="C1119" s="2" t="s">
-        <v>4362</v>
+        <v>4358</v>
       </c>
       <c r="D1119" s="2" t="s">
-        <v>97</v>
+        <v>205</v>
       </c>
       <c r="E1119" s="2" t="s">
-        <v>4363</v>
+        <v>4359</v>
       </c>
       <c r="F1119" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1119" s="3">
-        <v>22205</v>
-      </c>
+      <c r="G1119" s="2"/>
     </row>
     <row r="1120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1120" s="6" t="s">
-        <v>4364</v>
+        <v>4360</v>
       </c>
       <c r="B1120" s="2" t="s">
-        <v>4365</v>
+        <v>4361</v>
       </c>
       <c r="C1120" s="2" t="s">
-        <v>4366</v>
+        <v>4362</v>
       </c>
       <c r="D1120" s="2" t="s">
-        <v>313</v>
+        <v>97</v>
       </c>
       <c r="E1120" s="2" t="s">
-        <v>4367</v>
+        <v>4363</v>
       </c>
       <c r="F1120" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1120" s="2"/>
+      <c r="G1120" s="3">
+        <v>22205</v>
+      </c>
     </row>
     <row r="1121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1121" s="6" t="s">
-        <v>4368</v>
+        <v>4364</v>
       </c>
       <c r="B1121" s="2" t="s">
-        <v>4369</v>
+        <v>4365</v>
       </c>
       <c r="C1121" s="2" t="s">
-        <v>4370</v>
+        <v>4366</v>
       </c>
       <c r="D1121" s="2" t="s">
-        <v>4371</v>
+        <v>313</v>
       </c>
       <c r="E1121" s="2" t="s">
-        <v>4372</v>
+        <v>4367</v>
       </c>
       <c r="F1121" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1121" s="3">
-        <v>23369</v>
-      </c>
+      <c r="G1121" s="2"/>
     </row>
     <row r="1122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1122" s="6" t="s">
-        <v>4373</v>
+        <v>4368</v>
       </c>
       <c r="B1122" s="2" t="s">
-        <v>4374</v>
+        <v>4369</v>
       </c>
       <c r="C1122" s="2" t="s">
-        <v>4375</v>
+        <v>4370</v>
       </c>
       <c r="D1122" s="2" t="s">
-        <v>97</v>
+        <v>4371</v>
       </c>
       <c r="E1122" s="2" t="s">
-        <v>4376</v>
+        <v>4372</v>
       </c>
       <c r="F1122" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1122" s="3">
-        <v>19678</v>
+        <v>23369</v>
       </c>
     </row>
     <row r="1123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1123" s="6" t="s">
-        <v>4377</v>
+        <v>4373</v>
       </c>
       <c r="B1123" s="2" t="s">
-        <v>4378</v>
+        <v>4374</v>
       </c>
       <c r="C1123" s="2" t="s">
-        <v>1443</v>
+        <v>4375</v>
       </c>
       <c r="D1123" s="2" t="s">
-        <v>4379</v>
+        <v>97</v>
       </c>
       <c r="E1123" s="2" t="s">
-        <v>4380</v>
+        <v>4376</v>
       </c>
       <c r="F1123" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1123" s="2"/>
+      <c r="G1123" s="3">
+        <v>19678</v>
+      </c>
     </row>
     <row r="1124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1124" s="6" t="s">
-        <v>4381</v>
+        <v>4377</v>
       </c>
       <c r="B1124" s="2" t="s">
-        <v>4382</v>
+        <v>4378</v>
       </c>
       <c r="C1124" s="2" t="s">
-        <v>4383</v>
+        <v>1443</v>
       </c>
       <c r="D1124" s="2" t="s">
-        <v>1432</v>
+        <v>4379</v>
       </c>
       <c r="E1124" s="2" t="s">
-        <v>4384</v>
+        <v>4380</v>
       </c>
       <c r="F1124" s="2" t="s">
         <v>11</v>
@@ -39727,19 +39823,19 @@
     </row>
     <row r="1125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1125" s="6" t="s">
-        <v>4385</v>
+        <v>4381</v>
       </c>
       <c r="B1125" s="2" t="s">
-        <v>4386</v>
+        <v>4382</v>
       </c>
       <c r="C1125" s="2" t="s">
-        <v>4387</v>
+        <v>4383</v>
       </c>
       <c r="D1125" s="2" t="s">
-        <v>14</v>
+        <v>1432</v>
       </c>
       <c r="E1125" s="2" t="s">
-        <v>4388</v>
+        <v>4384</v>
       </c>
       <c r="F1125" s="2" t="s">
         <v>11</v>
@@ -39748,19 +39844,19 @@
     </row>
     <row r="1126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1126" s="6" t="s">
-        <v>4389</v>
+        <v>4385</v>
       </c>
       <c r="B1126" s="2" t="s">
-        <v>4390</v>
+        <v>4386</v>
       </c>
       <c r="C1126" s="2" t="s">
-        <v>4391</v>
+        <v>4387</v>
       </c>
       <c r="D1126" s="2" t="s">
-        <v>372</v>
+        <v>14</v>
       </c>
       <c r="E1126" s="2" t="s">
-        <v>4392</v>
+        <v>4388</v>
       </c>
       <c r="F1126" s="2" t="s">
         <v>11</v>
@@ -39769,241 +39865,241 @@
     </row>
     <row r="1127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1127" s="6" t="s">
-        <v>4393</v>
+        <v>4389</v>
       </c>
       <c r="B1127" s="2" t="s">
-        <v>4394</v>
+        <v>4390</v>
       </c>
       <c r="C1127" s="2" t="s">
-        <v>4395</v>
+        <v>4391</v>
       </c>
       <c r="D1127" s="2" t="s">
-        <v>109</v>
+        <v>372</v>
       </c>
       <c r="E1127" s="2" t="s">
-        <v>4396</v>
+        <v>4392</v>
       </c>
       <c r="F1127" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1127" s="3">
-        <v>8046</v>
-      </c>
+      <c r="G1127" s="2"/>
     </row>
     <row r="1128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1128" s="6" t="s">
-        <v>4397</v>
+        <v>4393</v>
       </c>
       <c r="B1128" s="2" t="s">
-        <v>4398</v>
+        <v>4394</v>
       </c>
       <c r="C1128" s="2" t="s">
-        <v>4399</v>
+        <v>4395</v>
       </c>
       <c r="D1128" s="2" t="s">
-        <v>274</v>
+        <v>109</v>
       </c>
       <c r="E1128" s="2" t="s">
-        <v>4400</v>
+        <v>4396</v>
       </c>
       <c r="F1128" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1128" s="3">
-        <v>22934</v>
+        <v>8046</v>
       </c>
     </row>
     <row r="1129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1129" s="6" t="s">
-        <v>4401</v>
+        <v>4397</v>
       </c>
       <c r="B1129" s="2" t="s">
-        <v>4402</v>
+        <v>4398</v>
       </c>
       <c r="C1129" s="2" t="s">
-        <v>4403</v>
+        <v>4399</v>
       </c>
       <c r="D1129" s="2" t="s">
-        <v>4404</v>
+        <v>274</v>
       </c>
       <c r="E1129" s="2" t="s">
-        <v>4405</v>
+        <v>4400</v>
       </c>
       <c r="F1129" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1129" s="3">
-        <v>29234</v>
+        <v>22934</v>
       </c>
     </row>
     <row r="1130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1130" s="6" t="s">
-        <v>4406</v>
-      </c>
-      <c r="B1130" s="2">
-        <v>885</v>
+        <v>4401</v>
+      </c>
+      <c r="B1130" s="2" t="s">
+        <v>4402</v>
       </c>
       <c r="C1130" s="2" t="s">
         <v>4403</v>
       </c>
       <c r="D1130" s="2" t="s">
-        <v>562</v>
+        <v>4404</v>
       </c>
       <c r="E1130" s="2" t="s">
-        <v>4407</v>
+        <v>4405</v>
       </c>
       <c r="F1130" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1130" s="2"/>
+      <c r="G1130" s="3">
+        <v>29234</v>
+      </c>
     </row>
     <row r="1131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1131" s="6" t="s">
-        <v>4408</v>
-      </c>
-      <c r="B1131" s="2" t="s">
-        <v>4409</v>
+        <v>4406</v>
+      </c>
+      <c r="B1131" s="2">
+        <v>885</v>
       </c>
       <c r="C1131" s="2" t="s">
-        <v>4410</v>
+        <v>4403</v>
       </c>
       <c r="D1131" s="2" t="s">
-        <v>318</v>
+        <v>562</v>
       </c>
       <c r="E1131" s="2" t="s">
-        <v>4411</v>
+        <v>4407</v>
       </c>
       <c r="F1131" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1131" s="3">
-        <v>6070</v>
-      </c>
+      <c r="G1131" s="2"/>
     </row>
     <row r="1132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1132" s="6" t="s">
-        <v>4412</v>
+        <v>4408</v>
       </c>
       <c r="B1132" s="2" t="s">
-        <v>4413</v>
+        <v>4409</v>
       </c>
       <c r="C1132" s="2" t="s">
         <v>4410</v>
       </c>
       <c r="D1132" s="2" t="s">
-        <v>215</v>
+        <v>318</v>
       </c>
       <c r="E1132" s="2" t="s">
-        <v>4414</v>
+        <v>4411</v>
       </c>
       <c r="F1132" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1132" s="3">
-        <v>32405</v>
+        <v>6070</v>
       </c>
     </row>
     <row r="1133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1133" s="6" t="s">
-        <v>4415</v>
+        <v>4412</v>
       </c>
       <c r="B1133" s="2" t="s">
-        <v>4416</v>
+        <v>4413</v>
       </c>
       <c r="C1133" s="2" t="s">
-        <v>4417</v>
+        <v>4410</v>
       </c>
       <c r="D1133" s="2" t="s">
-        <v>274</v>
+        <v>215</v>
       </c>
       <c r="E1133" s="2" t="s">
-        <v>4418</v>
+        <v>4414</v>
       </c>
       <c r="F1133" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1133" s="2"/>
+      <c r="G1133" s="3">
+        <v>32405</v>
+      </c>
     </row>
     <row r="1134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1134" s="6" t="s">
-        <v>4419</v>
+        <v>4415</v>
       </c>
       <c r="B1134" s="2" t="s">
-        <v>4420</v>
+        <v>4416</v>
       </c>
       <c r="C1134" s="2" t="s">
-        <v>4421</v>
+        <v>4417</v>
       </c>
       <c r="D1134" s="2" t="s">
-        <v>97</v>
+        <v>274</v>
       </c>
       <c r="E1134" s="2" t="s">
-        <v>4422</v>
+        <v>4418</v>
       </c>
       <c r="F1134" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1134" s="3">
-        <v>42030</v>
-      </c>
+      <c r="G1134" s="2"/>
     </row>
     <row r="1135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1135" s="6" t="s">
-        <v>4423</v>
+        <v>4419</v>
       </c>
       <c r="B1135" s="2" t="s">
-        <v>4424</v>
+        <v>4420</v>
       </c>
       <c r="C1135" s="2" t="s">
-        <v>4425</v>
+        <v>4421</v>
       </c>
       <c r="D1135" s="2" t="s">
-        <v>197</v>
+        <v>97</v>
       </c>
       <c r="E1135" s="2" t="s">
-        <v>4426</v>
+        <v>4422</v>
       </c>
       <c r="F1135" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1135" s="2"/>
+      <c r="G1135" s="3">
+        <v>42030</v>
+      </c>
     </row>
     <row r="1136" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1136" s="6" t="s">
-        <v>4427</v>
+        <v>4423</v>
       </c>
       <c r="B1136" s="2" t="s">
-        <v>4428</v>
+        <v>4424</v>
       </c>
       <c r="C1136" s="2" t="s">
-        <v>4429</v>
+        <v>4425</v>
       </c>
       <c r="D1136" s="2" t="s">
-        <v>4430</v>
+        <v>197</v>
       </c>
       <c r="E1136" s="2" t="s">
-        <v>4431</v>
+        <v>4426</v>
       </c>
       <c r="F1136" s="2" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="G1136" s="2"/>
     </row>
     <row r="1137" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1137" s="6" t="s">
-        <v>4432</v>
+        <v>4427</v>
       </c>
       <c r="B1137" s="2" t="s">
-        <v>4433</v>
+        <v>4428</v>
       </c>
       <c r="C1137" s="2" t="s">
-        <v>4434</v>
+        <v>4429</v>
       </c>
       <c r="D1137" s="2" t="s">
-        <v>1396</v>
+        <v>4430</v>
       </c>
       <c r="E1137" s="2" t="s">
-        <v>4435</v>
+        <v>4431</v>
       </c>
       <c r="F1137" s="2" t="s">
         <v>69</v>
@@ -40012,40 +40108,40 @@
     </row>
     <row r="1138" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1138" s="6" t="s">
-        <v>4436</v>
-      </c>
-      <c r="B1138" s="2">
-        <v>188315</v>
+        <v>4432</v>
+      </c>
+      <c r="B1138" s="2" t="s">
+        <v>4433</v>
       </c>
       <c r="C1138" s="2" t="s">
-        <v>4437</v>
+        <v>4434</v>
       </c>
       <c r="D1138" s="2" t="s">
-        <v>4438</v>
+        <v>1396</v>
       </c>
       <c r="E1138" s="2" t="s">
-        <v>4439</v>
+        <v>4435</v>
       </c>
       <c r="F1138" s="2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="G1138" s="2"/>
     </row>
     <row r="1139" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1139" s="6" t="s">
-        <v>4440</v>
+        <v>4436</v>
       </c>
       <c r="B1139" s="2">
-        <v>250077</v>
+        <v>188315</v>
       </c>
       <c r="C1139" s="2" t="s">
-        <v>4441</v>
+        <v>4437</v>
       </c>
       <c r="D1139" s="2" t="s">
-        <v>4442</v>
+        <v>4438</v>
       </c>
       <c r="E1139" s="2" t="s">
-        <v>4443</v>
+        <v>4439</v>
       </c>
       <c r="F1139" s="2" t="s">
         <v>11</v>
@@ -40054,19 +40150,19 @@
     </row>
     <row r="1140" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1140" s="6" t="s">
-        <v>4444</v>
-      </c>
-      <c r="B1140" s="2" t="s">
-        <v>4445</v>
+        <v>4440</v>
+      </c>
+      <c r="B1140" s="2">
+        <v>250077</v>
       </c>
       <c r="C1140" s="2" t="s">
-        <v>4446</v>
+        <v>4441</v>
       </c>
       <c r="D1140" s="2" t="s">
-        <v>735</v>
+        <v>4442</v>
       </c>
       <c r="E1140" s="2" t="s">
-        <v>4447</v>
+        <v>4443</v>
       </c>
       <c r="F1140" s="2" t="s">
         <v>11</v>
@@ -40075,19 +40171,19 @@
     </row>
     <row r="1141" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1141" s="6" t="s">
-        <v>4448</v>
+        <v>4444</v>
       </c>
       <c r="B1141" s="2" t="s">
-        <v>4449</v>
+        <v>4445</v>
       </c>
       <c r="C1141" s="2" t="s">
-        <v>4450</v>
+        <v>4446</v>
       </c>
       <c r="D1141" s="2" t="s">
-        <v>205</v>
+        <v>735</v>
       </c>
       <c r="E1141" s="2" t="s">
-        <v>4451</v>
+        <v>4447</v>
       </c>
       <c r="F1141" s="2" t="s">
         <v>11</v>
@@ -40096,19 +40192,19 @@
     </row>
     <row r="1142" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1142" s="6" t="s">
-        <v>4452</v>
+        <v>4448</v>
       </c>
       <c r="B1142" s="2" t="s">
-        <v>4453</v>
+        <v>4449</v>
       </c>
       <c r="C1142" s="2" t="s">
-        <v>4454</v>
+        <v>4450</v>
       </c>
       <c r="D1142" s="2" t="s">
-        <v>953</v>
+        <v>205</v>
       </c>
       <c r="E1142" s="2" t="s">
-        <v>4455</v>
+        <v>4451</v>
       </c>
       <c r="F1142" s="2" t="s">
         <v>11</v>
@@ -40117,167 +40213,165 @@
     </row>
     <row r="1143" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1143" s="6" t="s">
-        <v>4456</v>
+        <v>4452</v>
       </c>
       <c r="B1143" s="2" t="s">
-        <v>4457</v>
+        <v>4453</v>
       </c>
       <c r="C1143" s="2" t="s">
-        <v>4458</v>
+        <v>4454</v>
       </c>
       <c r="D1143" s="2" t="s">
-        <v>190</v>
+        <v>953</v>
       </c>
       <c r="E1143" s="2" t="s">
-        <v>4459</v>
+        <v>4455</v>
       </c>
       <c r="F1143" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1143" s="3">
-        <v>41072</v>
-      </c>
+      <c r="G1143" s="2"/>
     </row>
     <row r="1144" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1144" s="6" t="s">
-        <v>4460</v>
+        <v>4456</v>
       </c>
       <c r="B1144" s="2" t="s">
-        <v>4461</v>
+        <v>4457</v>
       </c>
       <c r="C1144" s="2" t="s">
-        <v>1556</v>
+        <v>4458</v>
       </c>
       <c r="D1144" s="2" t="s">
-        <v>45</v>
+        <v>190</v>
       </c>
       <c r="E1144" s="2" t="s">
-        <v>4462</v>
+        <v>4459</v>
       </c>
       <c r="F1144" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1144" s="3">
-        <v>7934</v>
+        <v>41072</v>
       </c>
     </row>
     <row r="1145" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1145" s="6" t="s">
-        <v>4463</v>
-      </c>
-      <c r="B1145" s="2">
-        <v>265967</v>
+        <v>4460</v>
+      </c>
+      <c r="B1145" s="2" t="s">
+        <v>4461</v>
       </c>
       <c r="C1145" s="2" t="s">
         <v>1556</v>
       </c>
       <c r="D1145" s="2" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="E1145" s="2" t="s">
-        <v>4464</v>
+        <v>4462</v>
       </c>
       <c r="F1145" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1145" s="2"/>
+      <c r="G1145" s="3">
+        <v>7934</v>
+      </c>
     </row>
     <row r="1146" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1146" s="6" t="s">
-        <v>4465</v>
-      </c>
-      <c r="B1146" s="2" t="s">
-        <v>4466</v>
+        <v>4463</v>
+      </c>
+      <c r="B1146" s="2">
+        <v>265967</v>
       </c>
       <c r="C1146" s="2" t="s">
-        <v>4467</v>
+        <v>1556</v>
       </c>
       <c r="D1146" s="2" t="s">
-        <v>1544</v>
+        <v>92</v>
       </c>
       <c r="E1146" s="2" t="s">
-        <v>4468</v>
+        <v>4464</v>
       </c>
       <c r="F1146" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1146" s="3">
-        <v>30691</v>
-      </c>
+      <c r="G1146" s="2"/>
     </row>
     <row r="1147" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1147" s="6" t="s">
-        <v>4469</v>
+        <v>4465</v>
       </c>
       <c r="B1147" s="2" t="s">
-        <v>4470</v>
+        <v>4466</v>
       </c>
       <c r="C1147" s="2" t="s">
-        <v>4471</v>
+        <v>4467</v>
       </c>
       <c r="D1147" s="2" t="s">
-        <v>125</v>
+        <v>1544</v>
       </c>
       <c r="E1147" s="2" t="s">
-        <v>4472</v>
+        <v>4468</v>
       </c>
       <c r="F1147" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1147" s="3">
-        <v>23223</v>
+        <v>30691</v>
       </c>
     </row>
     <row r="1148" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1148" s="6" t="s">
-        <v>4473</v>
+        <v>4469</v>
       </c>
       <c r="B1148" s="2" t="s">
-        <v>4474</v>
+        <v>4470</v>
       </c>
       <c r="C1148" s="2" t="s">
-        <v>4475</v>
+        <v>4471</v>
       </c>
       <c r="D1148" s="2" t="s">
-        <v>562</v>
+        <v>125</v>
       </c>
       <c r="E1148" s="2" t="s">
-        <v>4476</v>
+        <v>4472</v>
       </c>
       <c r="F1148" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1148" s="2"/>
+      <c r="G1148" s="3">
+        <v>23223</v>
+      </c>
     </row>
     <row r="1149" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1149" s="6" t="s">
-        <v>4477</v>
+        <v>4473</v>
       </c>
       <c r="B1149" s="2" t="s">
-        <v>4478</v>
+        <v>4474</v>
       </c>
       <c r="C1149" s="2" t="s">
-        <v>4479</v>
+        <v>4475</v>
       </c>
       <c r="D1149" s="2" t="s">
-        <v>313</v>
+        <v>562</v>
       </c>
       <c r="E1149" s="2" t="s">
-        <v>4480</v>
+        <v>4476</v>
       </c>
       <c r="F1149" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1149" s="3">
-        <v>12882</v>
-      </c>
+      <c r="G1149" s="2"/>
     </row>
     <row r="1150" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1150" s="6" t="s">
-        <v>4481</v>
+        <v>4477</v>
       </c>
       <c r="B1150" s="2" t="s">
-        <v>4482</v>
+        <v>4478</v>
       </c>
       <c r="C1150" s="2" t="s">
         <v>4479</v>
@@ -40286,652 +40380,654 @@
         <v>313</v>
       </c>
       <c r="E1150" s="2" t="s">
-        <v>4483</v>
+        <v>4480</v>
       </c>
       <c r="F1150" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1150" s="3">
-        <v>26284</v>
+        <v>12882</v>
       </c>
     </row>
     <row r="1151" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1151" s="6" t="s">
-        <v>4484</v>
+        <v>4481</v>
       </c>
       <c r="B1151" s="2" t="s">
-        <v>4485</v>
+        <v>4482</v>
       </c>
       <c r="C1151" s="2" t="s">
-        <v>4486</v>
+        <v>4479</v>
       </c>
       <c r="D1151" s="2" t="s">
-        <v>132</v>
+        <v>313</v>
       </c>
       <c r="E1151" s="2" t="s">
-        <v>4487</v>
+        <v>4483</v>
       </c>
       <c r="F1151" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1151" s="3">
-        <v>14235</v>
+        <v>26284</v>
       </c>
     </row>
     <row r="1152" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1152" s="6" t="s">
-        <v>4488</v>
+        <v>4484</v>
       </c>
       <c r="B1152" s="2" t="s">
-        <v>4489</v>
+        <v>4485</v>
       </c>
       <c r="C1152" s="2" t="s">
         <v>4486</v>
       </c>
       <c r="D1152" s="2" t="s">
-        <v>27</v>
+        <v>132</v>
       </c>
       <c r="E1152" s="2" t="s">
-        <v>4490</v>
+        <v>4487</v>
       </c>
       <c r="F1152" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1152" s="3">
-        <v>15298</v>
+        <v>14235</v>
       </c>
     </row>
     <row r="1153" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1153" s="6" t="s">
-        <v>4491</v>
+        <v>4488</v>
       </c>
       <c r="B1153" s="2" t="s">
-        <v>4492</v>
+        <v>4489</v>
       </c>
       <c r="C1153" s="2" t="s">
         <v>4486</v>
       </c>
       <c r="D1153" s="2" t="s">
-        <v>313</v>
+        <v>27</v>
       </c>
       <c r="E1153" s="2" t="s">
-        <v>4493</v>
+        <v>4490</v>
       </c>
       <c r="F1153" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1153" s="2"/>
+      <c r="G1153" s="3">
+        <v>15298</v>
+      </c>
     </row>
     <row r="1154" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1154" s="6" t="s">
-        <v>4494</v>
+        <v>4491</v>
       </c>
       <c r="B1154" s="2" t="s">
-        <v>4495</v>
+        <v>4492</v>
       </c>
       <c r="C1154" s="2" t="s">
-        <v>4496</v>
+        <v>4486</v>
       </c>
       <c r="D1154" s="2" t="s">
-        <v>132</v>
+        <v>313</v>
       </c>
       <c r="E1154" s="2" t="s">
-        <v>4497</v>
+        <v>4493</v>
       </c>
       <c r="F1154" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1154" s="3">
-        <v>17058</v>
-      </c>
+      <c r="G1154" s="2"/>
     </row>
     <row r="1155" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1155" s="6" t="s">
-        <v>4498</v>
-      </c>
-      <c r="B1155" s="2">
-        <v>193430</v>
+        <v>4494</v>
+      </c>
+      <c r="B1155" s="2" t="s">
+        <v>4495</v>
       </c>
       <c r="C1155" s="2" t="s">
-        <v>4499</v>
+        <v>4496</v>
       </c>
       <c r="D1155" s="2" t="s">
-        <v>1569</v>
+        <v>132</v>
       </c>
       <c r="E1155" s="2" t="s">
-        <v>4500</v>
+        <v>4497</v>
       </c>
       <c r="F1155" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1155" s="2"/>
+      <c r="G1155" s="3">
+        <v>17058</v>
+      </c>
     </row>
     <row r="1156" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1156" s="6" t="s">
-        <v>4501</v>
-      </c>
-      <c r="B1156" s="2" t="s">
-        <v>4502</v>
+        <v>4498</v>
+      </c>
+      <c r="B1156" s="2">
+        <v>193430</v>
       </c>
       <c r="C1156" s="2" t="s">
-        <v>4503</v>
+        <v>4499</v>
       </c>
       <c r="D1156" s="2" t="s">
-        <v>14</v>
+        <v>1569</v>
       </c>
       <c r="E1156" s="2" t="s">
-        <v>4504</v>
+        <v>4500</v>
       </c>
       <c r="F1156" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1156" s="3">
-        <v>36845</v>
-      </c>
+      <c r="G1156" s="2"/>
     </row>
     <row r="1157" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1157" s="6" t="s">
-        <v>4505</v>
+        <v>4501</v>
       </c>
       <c r="B1157" s="2" t="s">
-        <v>4506</v>
+        <v>4502</v>
       </c>
       <c r="C1157" s="2" t="s">
-        <v>4507</v>
+        <v>4503</v>
       </c>
       <c r="D1157" s="2" t="s">
-        <v>132</v>
+        <v>14</v>
       </c>
       <c r="E1157" s="2" t="s">
-        <v>4508</v>
+        <v>4504</v>
       </c>
       <c r="F1157" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1157" s="3">
-        <v>13433</v>
+        <v>36845</v>
       </c>
     </row>
     <row r="1158" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1158" s="6" t="s">
-        <v>4509</v>
+        <v>4505</v>
       </c>
       <c r="B1158" s="2" t="s">
-        <v>4510</v>
+        <v>4506</v>
       </c>
       <c r="C1158" s="2" t="s">
         <v>4507</v>
       </c>
       <c r="D1158" s="2" t="s">
-        <v>4511</v>
+        <v>132</v>
       </c>
       <c r="E1158" s="2" t="s">
-        <v>4512</v>
+        <v>4508</v>
       </c>
       <c r="F1158" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1158" s="2"/>
+      <c r="G1158" s="3">
+        <v>13433</v>
+      </c>
     </row>
     <row r="1159" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1159" s="6" t="s">
-        <v>4513</v>
-      </c>
-      <c r="B1159" s="2">
-        <v>281688</v>
+        <v>4509</v>
+      </c>
+      <c r="B1159" s="2" t="s">
+        <v>4510</v>
       </c>
       <c r="C1159" s="2" t="s">
         <v>4507</v>
       </c>
       <c r="D1159" s="2" t="s">
-        <v>72</v>
+        <v>4511</v>
       </c>
       <c r="E1159" s="2" t="s">
-        <v>4514</v>
+        <v>4512</v>
       </c>
       <c r="F1159" s="2" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="G1159" s="2"/>
     </row>
     <row r="1160" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1160" s="6" t="s">
-        <v>4515</v>
-      </c>
-      <c r="B1160" s="2" t="s">
-        <v>4516</v>
+        <v>4513</v>
+      </c>
+      <c r="B1160" s="2">
+        <v>281688</v>
       </c>
       <c r="C1160" s="2" t="s">
-        <v>4517</v>
+        <v>4507</v>
       </c>
       <c r="D1160" s="2" t="s">
-        <v>4518</v>
+        <v>72</v>
       </c>
       <c r="E1160" s="2" t="s">
-        <v>4519</v>
+        <v>4514</v>
       </c>
       <c r="F1160" s="2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="G1160" s="2"/>
     </row>
     <row r="1161" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1161" s="6" t="s">
-        <v>4520</v>
-      </c>
-      <c r="B1161" s="2">
-        <v>264121</v>
+        <v>4515</v>
+      </c>
+      <c r="B1161" s="2" t="s">
+        <v>4516</v>
       </c>
       <c r="C1161" s="2" t="s">
         <v>4517</v>
       </c>
       <c r="D1161" s="2" t="s">
-        <v>4521</v>
+        <v>4518</v>
       </c>
       <c r="E1161" s="2" t="s">
-        <v>4522</v>
+        <v>4519</v>
       </c>
       <c r="F1161" s="2" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="G1161" s="2"/>
     </row>
     <row r="1162" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1162" s="6" t="s">
-        <v>4523</v>
-      </c>
-      <c r="B1162" s="2" t="s">
-        <v>4524</v>
+        <v>4520</v>
+      </c>
+      <c r="B1162" s="2">
+        <v>264121</v>
       </c>
       <c r="C1162" s="2" t="s">
-        <v>4525</v>
+        <v>4517</v>
       </c>
       <c r="D1162" s="2" t="s">
-        <v>132</v>
+        <v>4521</v>
       </c>
       <c r="E1162" s="2" t="s">
-        <v>4526</v>
+        <v>4522</v>
       </c>
       <c r="F1162" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1162" s="3">
-        <v>37787</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="G1162" s="2"/>
     </row>
     <row r="1163" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1163" s="6" t="s">
-        <v>4527</v>
+        <v>4523</v>
       </c>
       <c r="B1163" s="2" t="s">
-        <v>4528</v>
+        <v>4524</v>
       </c>
       <c r="C1163" s="2" t="s">
-        <v>4529</v>
+        <v>4525</v>
       </c>
       <c r="D1163" s="2" t="s">
-        <v>27</v>
+        <v>132</v>
       </c>
       <c r="E1163" s="2" t="s">
-        <v>4530</v>
+        <v>4526</v>
       </c>
       <c r="F1163" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1163" s="3">
-        <v>11359</v>
+        <v>37787</v>
       </c>
     </row>
     <row r="1164" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1164" s="6" t="s">
-        <v>4531</v>
+        <v>4527</v>
       </c>
       <c r="B1164" s="2" t="s">
-        <v>4532</v>
+        <v>4528</v>
       </c>
       <c r="C1164" s="2" t="s">
         <v>4529</v>
       </c>
       <c r="D1164" s="2" t="s">
-        <v>4193</v>
+        <v>27</v>
       </c>
       <c r="E1164" s="2" t="s">
-        <v>4533</v>
+        <v>4530</v>
       </c>
       <c r="F1164" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1164" s="2"/>
+      <c r="G1164" s="3">
+        <v>11359</v>
+      </c>
     </row>
     <row r="1165" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1165" s="6" t="s">
-        <v>4534</v>
+        <v>4531</v>
       </c>
       <c r="B1165" s="2" t="s">
-        <v>4535</v>
+        <v>4532</v>
       </c>
       <c r="C1165" s="2" t="s">
         <v>4529</v>
       </c>
       <c r="D1165" s="2" t="s">
-        <v>4536</v>
+        <v>4193</v>
       </c>
       <c r="E1165" s="2" t="s">
-        <v>4537</v>
+        <v>4533</v>
       </c>
       <c r="F1165" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1165" s="3">
-        <v>40288</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="G1165" s="2"/>
     </row>
     <row r="1166" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1166" s="6" t="s">
-        <v>4538</v>
+        <v>4534</v>
       </c>
       <c r="B1166" s="2" t="s">
-        <v>4539</v>
+        <v>4535</v>
       </c>
       <c r="C1166" s="2" t="s">
-        <v>4540</v>
+        <v>4529</v>
       </c>
       <c r="D1166" s="2" t="s">
-        <v>205</v>
+        <v>4536</v>
       </c>
       <c r="E1166" s="2" t="s">
-        <v>4541</v>
+        <v>4537</v>
       </c>
       <c r="F1166" s="2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="G1166" s="3">
-        <v>42281</v>
+        <v>40288</v>
       </c>
     </row>
     <row r="1167" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1167" s="6" t="s">
-        <v>4542</v>
+        <v>4538</v>
       </c>
       <c r="B1167" s="2" t="s">
-        <v>4543</v>
+        <v>4539</v>
       </c>
       <c r="C1167" s="2" t="s">
-        <v>4544</v>
+        <v>4540</v>
       </c>
       <c r="D1167" s="2" t="s">
-        <v>3872</v>
+        <v>205</v>
       </c>
       <c r="E1167" s="2" t="s">
-        <v>4545</v>
+        <v>4541</v>
       </c>
       <c r="F1167" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1167" s="3">
-        <v>26008</v>
+        <v>42281</v>
       </c>
     </row>
     <row r="1168" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1168" s="6" t="s">
-        <v>4546</v>
+        <v>4542</v>
       </c>
       <c r="B1168" s="2" t="s">
-        <v>4547</v>
+        <v>4543</v>
       </c>
       <c r="C1168" s="2" t="s">
-        <v>4548</v>
+        <v>4544</v>
       </c>
       <c r="D1168" s="2" t="s">
-        <v>97</v>
+        <v>3872</v>
       </c>
       <c r="E1168" s="2" t="s">
-        <v>4549</v>
+        <v>4545</v>
       </c>
       <c r="F1168" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1168" s="3">
-        <v>21106</v>
+        <v>26008</v>
       </c>
     </row>
     <row r="1169" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1169" s="6" t="s">
-        <v>4550</v>
+        <v>4546</v>
       </c>
       <c r="B1169" s="2" t="s">
-        <v>4551</v>
+        <v>4547</v>
       </c>
       <c r="C1169" s="2" t="s">
         <v>4548</v>
       </c>
       <c r="D1169" s="2" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E1169" s="2" t="s">
-        <v>4552</v>
+        <v>4549</v>
       </c>
       <c r="F1169" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1169" s="3">
-        <v>38396</v>
+        <v>21106</v>
       </c>
     </row>
     <row r="1170" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1170" s="6" t="s">
-        <v>4553</v>
-      </c>
-      <c r="B1170" s="2">
-        <v>207800</v>
+        <v>4550</v>
+      </c>
+      <c r="B1170" s="2" t="s">
+        <v>4551</v>
       </c>
       <c r="C1170" s="2" t="s">
-        <v>4554</v>
+        <v>4548</v>
       </c>
       <c r="D1170" s="2" t="s">
-        <v>3736</v>
+        <v>88</v>
       </c>
       <c r="E1170" s="2" t="s">
-        <v>4555</v>
+        <v>4552</v>
       </c>
       <c r="F1170" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1170" s="2"/>
+      <c r="G1170" s="3">
+        <v>38396</v>
+      </c>
     </row>
     <row r="1171" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1171" s="6" t="s">
-        <v>4556</v>
-      </c>
-      <c r="B1171" s="2" t="s">
-        <v>4557</v>
+        <v>4553</v>
+      </c>
+      <c r="B1171" s="2">
+        <v>207800</v>
       </c>
       <c r="C1171" s="2" t="s">
-        <v>4558</v>
+        <v>4554</v>
       </c>
       <c r="D1171" s="2" t="s">
-        <v>125</v>
+        <v>3736</v>
       </c>
       <c r="E1171" s="2" t="s">
-        <v>4559</v>
+        <v>4555</v>
       </c>
       <c r="F1171" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1171" s="3">
-        <v>41933</v>
-      </c>
+      <c r="G1171" s="2"/>
     </row>
     <row r="1172" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1172" s="6" t="s">
-        <v>4560</v>
+        <v>4556</v>
       </c>
       <c r="B1172" s="2" t="s">
-        <v>4561</v>
+        <v>4557</v>
       </c>
       <c r="C1172" s="2" t="s">
         <v>4558</v>
       </c>
       <c r="D1172" s="2" t="s">
-        <v>2700</v>
+        <v>125</v>
       </c>
       <c r="E1172" s="2" t="s">
-        <v>4562</v>
+        <v>4559</v>
       </c>
       <c r="F1172" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1172" s="2"/>
+      <c r="G1172" s="3">
+        <v>41933</v>
+      </c>
     </row>
     <row r="1173" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1173" s="6" t="s">
-        <v>4563</v>
+        <v>4560</v>
       </c>
       <c r="B1173" s="2" t="s">
-        <v>4564</v>
+        <v>4561</v>
       </c>
       <c r="C1173" s="2" t="s">
-        <v>4565</v>
+        <v>4558</v>
       </c>
       <c r="D1173" s="2" t="s">
-        <v>654</v>
+        <v>2700</v>
       </c>
       <c r="E1173" s="2" t="s">
-        <v>4566</v>
+        <v>4562</v>
       </c>
       <c r="F1173" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1173" s="3">
-        <v>15963</v>
-      </c>
+      <c r="G1173" s="2"/>
     </row>
     <row r="1174" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1174" s="6" t="s">
-        <v>4567</v>
+        <v>4563</v>
       </c>
       <c r="B1174" s="2" t="s">
-        <v>4568</v>
+        <v>4564</v>
       </c>
       <c r="C1174" s="2" t="s">
-        <v>4569</v>
+        <v>4565</v>
       </c>
       <c r="D1174" s="2" t="s">
-        <v>513</v>
+        <v>654</v>
       </c>
       <c r="E1174" s="2" t="s">
-        <v>4570</v>
+        <v>4566</v>
       </c>
       <c r="F1174" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1174" s="3">
-        <v>34921</v>
+        <v>15963</v>
       </c>
     </row>
     <row r="1175" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1175" s="6" t="s">
-        <v>4571</v>
-      </c>
-      <c r="B1175" s="2">
-        <v>241590</v>
+        <v>4567</v>
+      </c>
+      <c r="B1175" s="2" t="s">
+        <v>4568</v>
       </c>
       <c r="C1175" s="2" t="s">
-        <v>4572</v>
+        <v>4569</v>
       </c>
       <c r="D1175" s="2" t="s">
-        <v>4573</v>
+        <v>513</v>
       </c>
       <c r="E1175" s="2" t="s">
-        <v>4574</v>
+        <v>4570</v>
       </c>
       <c r="F1175" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1175" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="G1175" s="3">
+        <v>34921</v>
+      </c>
     </row>
     <row r="1176" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1176" s="6" t="s">
-        <v>4575</v>
-      </c>
-      <c r="B1176" s="2" t="s">
-        <v>4576</v>
+        <v>4571</v>
+      </c>
+      <c r="B1176" s="2">
+        <v>241590</v>
       </c>
       <c r="C1176" s="2" t="s">
-        <v>4577</v>
+        <v>4572</v>
       </c>
       <c r="D1176" s="2" t="s">
-        <v>4578</v>
+        <v>4573</v>
       </c>
       <c r="E1176" s="2" t="s">
-        <v>4579</v>
+        <v>4574</v>
       </c>
       <c r="F1176" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1176" s="3">
-        <v>14864</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="G1176" s="2"/>
     </row>
     <row r="1177" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1177" s="6" t="s">
-        <v>4580</v>
+        <v>4575</v>
       </c>
       <c r="B1177" s="2" t="s">
-        <v>4581</v>
+        <v>4576</v>
       </c>
       <c r="C1177" s="2" t="s">
-        <v>4582</v>
+        <v>4577</v>
       </c>
       <c r="D1177" s="2" t="s">
-        <v>185</v>
+        <v>4578</v>
       </c>
       <c r="E1177" s="2" t="s">
-        <v>4583</v>
+        <v>4579</v>
       </c>
       <c r="F1177" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1177" s="3">
-        <v>25236</v>
+        <v>14864</v>
       </c>
     </row>
     <row r="1178" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1178" s="6" t="s">
-        <v>4584</v>
+        <v>4580</v>
       </c>
       <c r="B1178" s="2" t="s">
-        <v>4585</v>
+        <v>4581</v>
       </c>
       <c r="C1178" s="2" t="s">
-        <v>4586</v>
+        <v>4582</v>
       </c>
       <c r="D1178" s="2" t="s">
-        <v>301</v>
+        <v>185</v>
       </c>
       <c r="E1178" s="2" t="s">
-        <v>4587</v>
+        <v>4583</v>
       </c>
       <c r="F1178" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1178" s="2"/>
+      <c r="G1178" s="3">
+        <v>25236</v>
+      </c>
     </row>
     <row r="1179" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1179" s="6" t="s">
-        <v>4588</v>
+        <v>4584</v>
       </c>
       <c r="B1179" s="2" t="s">
-        <v>4589</v>
+        <v>4585</v>
       </c>
       <c r="C1179" s="2" t="s">
         <v>4586</v>
       </c>
       <c r="D1179" s="2" t="s">
-        <v>92</v>
+        <v>301</v>
       </c>
       <c r="E1179" s="2" t="s">
-        <v>4590</v>
+        <v>4587</v>
       </c>
       <c r="F1179" s="2" t="s">
         <v>11</v>
@@ -40940,109 +41036,109 @@
     </row>
     <row r="1180" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1180" s="6" t="s">
-        <v>4591</v>
+        <v>4588</v>
       </c>
       <c r="B1180" s="2" t="s">
-        <v>4592</v>
+        <v>4589</v>
       </c>
       <c r="C1180" s="2" t="s">
-        <v>4593</v>
+        <v>4586</v>
       </c>
       <c r="D1180" s="2" t="s">
-        <v>274</v>
+        <v>92</v>
       </c>
       <c r="E1180" s="2" t="s">
-        <v>4594</v>
+        <v>4590</v>
       </c>
       <c r="F1180" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1180" s="3">
-        <v>5490</v>
-      </c>
+      <c r="G1180" s="2"/>
     </row>
     <row r="1181" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1181" s="6" t="s">
-        <v>4595</v>
+        <v>4591</v>
       </c>
       <c r="B1181" s="2" t="s">
-        <v>4596</v>
+        <v>4592</v>
       </c>
       <c r="C1181" s="2" t="s">
-        <v>4597</v>
+        <v>4593</v>
       </c>
       <c r="D1181" s="2" t="s">
-        <v>132</v>
+        <v>274</v>
       </c>
       <c r="E1181" s="2" t="s">
-        <v>4598</v>
+        <v>4594</v>
       </c>
       <c r="F1181" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1181" s="3">
-        <v>14646</v>
+        <v>5490</v>
       </c>
     </row>
     <row r="1182" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1182" s="6" t="s">
-        <v>4599</v>
+        <v>4595</v>
       </c>
       <c r="B1182" s="2" t="s">
-        <v>4600</v>
+        <v>4596</v>
       </c>
       <c r="C1182" s="2" t="s">
-        <v>4601</v>
+        <v>4597</v>
       </c>
       <c r="D1182" s="2" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="E1182" s="2" t="s">
-        <v>4602</v>
+        <v>4598</v>
       </c>
       <c r="F1182" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1182" s="3">
-        <v>33759</v>
+        <v>14646</v>
       </c>
     </row>
     <row r="1183" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1183" s="6" t="s">
-        <v>4603</v>
+        <v>4599</v>
       </c>
       <c r="B1183" s="2" t="s">
-        <v>4604</v>
+        <v>4600</v>
       </c>
       <c r="C1183" s="2" t="s">
         <v>4601</v>
       </c>
       <c r="D1183" s="2" t="s">
-        <v>3257</v>
+        <v>97</v>
       </c>
       <c r="E1183" s="2" t="s">
-        <v>4605</v>
+        <v>4602</v>
       </c>
       <c r="F1183" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1183" s="2"/>
+      <c r="G1183" s="3">
+        <v>33759</v>
+      </c>
     </row>
     <row r="1184" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1184" s="6" t="s">
-        <v>4606</v>
-      </c>
-      <c r="B1184" s="2">
-        <v>249758</v>
+        <v>4603</v>
+      </c>
+      <c r="B1184" s="2" t="s">
+        <v>4604</v>
       </c>
       <c r="C1184" s="2" t="s">
         <v>4601</v>
       </c>
       <c r="D1184" s="2" t="s">
-        <v>845</v>
+        <v>3257</v>
       </c>
       <c r="E1184" s="2" t="s">
-        <v>4607</v>
+        <v>4605</v>
       </c>
       <c r="F1184" s="2" t="s">
         <v>11</v>
@@ -41051,176 +41147,176 @@
     </row>
     <row r="1185" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1185" s="6" t="s">
-        <v>4608</v>
-      </c>
-      <c r="B1185" s="2" t="s">
-        <v>4609</v>
+        <v>4606</v>
+      </c>
+      <c r="B1185" s="2">
+        <v>249758</v>
       </c>
       <c r="C1185" s="2" t="s">
-        <v>4610</v>
+        <v>4601</v>
       </c>
       <c r="D1185" s="2" t="s">
-        <v>215</v>
+        <v>845</v>
       </c>
       <c r="E1185" s="2" t="s">
-        <v>4611</v>
+        <v>4607</v>
       </c>
       <c r="F1185" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1185" s="3">
-        <v>18317</v>
-      </c>
+      <c r="G1185" s="2"/>
     </row>
     <row r="1186" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1186" s="6" t="s">
-        <v>4612</v>
+        <v>4608</v>
       </c>
       <c r="B1186" s="2" t="s">
-        <v>4613</v>
+        <v>4609</v>
       </c>
       <c r="C1186" s="2" t="s">
         <v>4610</v>
       </c>
       <c r="D1186" s="2" t="s">
-        <v>2318</v>
+        <v>215</v>
       </c>
       <c r="E1186" s="2" t="s">
-        <v>4614</v>
+        <v>4611</v>
       </c>
       <c r="F1186" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1186" s="2"/>
+      <c r="G1186" s="3">
+        <v>18317</v>
+      </c>
     </row>
     <row r="1187" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1187" s="6" t="s">
-        <v>4615</v>
+        <v>4612</v>
       </c>
       <c r="B1187" s="2" t="s">
-        <v>4616</v>
+        <v>4613</v>
       </c>
       <c r="C1187" s="2" t="s">
-        <v>4617</v>
+        <v>4610</v>
       </c>
       <c r="D1187" s="2" t="s">
-        <v>27</v>
+        <v>2318</v>
       </c>
       <c r="E1187" s="2" t="s">
-        <v>4618</v>
+        <v>4614</v>
       </c>
       <c r="F1187" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1187" s="3">
-        <v>17765</v>
-      </c>
+      <c r="G1187" s="2"/>
     </row>
     <row r="1188" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1188" s="6" t="s">
-        <v>4619</v>
+        <v>4615</v>
       </c>
       <c r="B1188" s="2" t="s">
-        <v>4620</v>
+        <v>4616</v>
       </c>
       <c r="C1188" s="2" t="s">
         <v>4617</v>
       </c>
       <c r="D1188" s="2" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="E1188" s="2" t="s">
-        <v>4621</v>
+        <v>4618</v>
       </c>
       <c r="F1188" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1188" s="3">
-        <v>19750</v>
+        <v>17765</v>
       </c>
     </row>
     <row r="1189" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1189" s="6" t="s">
-        <v>4622</v>
+        <v>4619</v>
       </c>
       <c r="B1189" s="2" t="s">
-        <v>4623</v>
+        <v>4620</v>
       </c>
       <c r="C1189" s="2" t="s">
         <v>4617</v>
       </c>
       <c r="D1189" s="2" t="s">
-        <v>1467</v>
+        <v>58</v>
       </c>
       <c r="E1189" s="2" t="s">
-        <v>4624</v>
+        <v>4621</v>
       </c>
       <c r="F1189" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1189" s="3">
-        <v>32048</v>
+        <v>19750</v>
       </c>
     </row>
     <row r="1190" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1190" s="6" t="s">
-        <v>4625</v>
+        <v>4622</v>
       </c>
       <c r="B1190" s="2" t="s">
-        <v>4626</v>
+        <v>4623</v>
       </c>
       <c r="C1190" s="2" t="s">
         <v>4617</v>
       </c>
       <c r="D1190" s="2" t="s">
-        <v>728</v>
+        <v>1467</v>
       </c>
       <c r="E1190" s="2" t="s">
-        <v>4627</v>
+        <v>4624</v>
       </c>
       <c r="F1190" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1190" s="3">
-        <v>41366</v>
+        <v>32048</v>
       </c>
     </row>
     <row r="1191" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1191" s="6" t="s">
-        <v>4628</v>
-      </c>
-      <c r="B1191" s="2">
-        <v>198084</v>
+        <v>4625</v>
+      </c>
+      <c r="B1191" s="2" t="s">
+        <v>4626</v>
       </c>
       <c r="C1191" s="2" t="s">
         <v>4617</v>
       </c>
       <c r="D1191" s="2" t="s">
-        <v>775</v>
+        <v>728</v>
       </c>
       <c r="E1191" s="2" t="s">
-        <v>4629</v>
+        <v>4627</v>
       </c>
       <c r="F1191" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1191" s="2"/>
+      <c r="G1191" s="3">
+        <v>41366</v>
+      </c>
     </row>
     <row r="1192" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1192" s="6" t="s">
-        <v>4630</v>
+        <v>4628</v>
       </c>
       <c r="B1192" s="2">
-        <v>265970</v>
+        <v>198084</v>
       </c>
       <c r="C1192" s="2" t="s">
         <v>4617</v>
       </c>
       <c r="D1192" s="2" t="s">
-        <v>654</v>
+        <v>775</v>
       </c>
       <c r="E1192" s="2" t="s">
-        <v>4631</v>
+        <v>4629</v>
       </c>
       <c r="F1192" s="2" t="s">
         <v>11</v>
@@ -41229,19 +41325,19 @@
     </row>
     <row r="1193" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1193" s="6" t="s">
-        <v>4632</v>
-      </c>
-      <c r="B1193" s="2" t="s">
-        <v>4633</v>
+        <v>4630</v>
+      </c>
+      <c r="B1193" s="2">
+        <v>265970</v>
       </c>
       <c r="C1193" s="2" t="s">
         <v>4617</v>
       </c>
       <c r="D1193" s="2" t="s">
-        <v>1569</v>
+        <v>654</v>
       </c>
       <c r="E1193" s="2" t="s">
-        <v>4634</v>
+        <v>4631</v>
       </c>
       <c r="F1193" s="2" t="s">
         <v>11</v>
@@ -41250,107 +41346,107 @@
     </row>
     <row r="1194" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1194" s="6" t="s">
-        <v>4635</v>
+        <v>4632</v>
       </c>
       <c r="B1194" s="2" t="s">
-        <v>4636</v>
+        <v>4633</v>
       </c>
       <c r="C1194" s="2" t="s">
-        <v>4637</v>
+        <v>4617</v>
       </c>
       <c r="D1194" s="2" t="s">
-        <v>994</v>
+        <v>1569</v>
       </c>
       <c r="E1194" s="2" t="s">
-        <v>4638</v>
+        <v>4634</v>
       </c>
       <c r="F1194" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1194" s="3">
-        <v>36691</v>
-      </c>
+      <c r="G1194" s="2"/>
     </row>
     <row r="1195" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1195" s="6" t="s">
-        <v>4639</v>
+        <v>4635</v>
       </c>
       <c r="B1195" s="2" t="s">
-        <v>4640</v>
+        <v>4636</v>
       </c>
       <c r="C1195" s="2" t="s">
-        <v>4641</v>
+        <v>4637</v>
       </c>
       <c r="D1195" s="2" t="s">
-        <v>2700</v>
+        <v>994</v>
       </c>
       <c r="E1195" s="2" t="s">
-        <v>4642</v>
+        <v>4638</v>
       </c>
       <c r="F1195" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1195" s="2"/>
+      <c r="G1195" s="3">
+        <v>36691</v>
+      </c>
     </row>
     <row r="1196" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1196" s="6" t="s">
-        <v>4643</v>
+        <v>4639</v>
       </c>
       <c r="B1196" s="2" t="s">
-        <v>4644</v>
+        <v>4640</v>
       </c>
       <c r="C1196" s="2" t="s">
-        <v>4645</v>
+        <v>4641</v>
       </c>
       <c r="D1196" s="2" t="s">
-        <v>318</v>
+        <v>2700</v>
       </c>
       <c r="E1196" s="2" t="s">
-        <v>4646</v>
+        <v>4642</v>
       </c>
       <c r="F1196" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1196" s="3">
-        <v>18475</v>
-      </c>
+      <c r="G1196" s="2"/>
     </row>
     <row r="1197" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1197" s="6" t="s">
-        <v>4647</v>
+        <v>4643</v>
       </c>
       <c r="B1197" s="2" t="s">
-        <v>4648</v>
+        <v>4644</v>
       </c>
       <c r="C1197" s="2" t="s">
-        <v>4649</v>
+        <v>4645</v>
       </c>
       <c r="D1197" s="2" t="s">
-        <v>892</v>
+        <v>318</v>
       </c>
       <c r="E1197" s="2" t="s">
-        <v>4650</v>
+        <v>4646</v>
       </c>
       <c r="F1197" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1197" s="2"/>
+      <c r="G1197" s="3">
+        <v>18475</v>
+      </c>
     </row>
     <row r="1198" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1198" s="6" t="s">
-        <v>4651</v>
+        <v>4647</v>
       </c>
       <c r="B1198" s="2" t="s">
-        <v>4652</v>
+        <v>4648</v>
       </c>
       <c r="C1198" s="2" t="s">
-        <v>4653</v>
+        <v>4649</v>
       </c>
       <c r="D1198" s="2" t="s">
-        <v>3731</v>
+        <v>892</v>
       </c>
       <c r="E1198" s="2" t="s">
-        <v>4654</v>
+        <v>4650</v>
       </c>
       <c r="F1198" s="2" t="s">
         <v>11</v>
@@ -41359,19 +41455,19 @@
     </row>
     <row r="1199" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1199" s="6" t="s">
-        <v>4655</v>
+        <v>4651</v>
       </c>
       <c r="B1199" s="2" t="s">
-        <v>4656</v>
+        <v>4652</v>
       </c>
       <c r="C1199" s="2" t="s">
         <v>4653</v>
       </c>
       <c r="D1199" s="2" t="s">
-        <v>205</v>
+        <v>3731</v>
       </c>
       <c r="E1199" s="2" t="s">
-        <v>4657</v>
+        <v>4654</v>
       </c>
       <c r="F1199" s="2" t="s">
         <v>11</v>
@@ -41380,19 +41476,19 @@
     </row>
     <row r="1200" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1200" s="6" t="s">
-        <v>4658</v>
-      </c>
-      <c r="B1200" s="4">
-        <v>80000</v>
+        <v>4655</v>
+      </c>
+      <c r="B1200" s="2" t="s">
+        <v>4656</v>
       </c>
       <c r="C1200" s="2" t="s">
-        <v>4659</v>
+        <v>4653</v>
       </c>
       <c r="D1200" s="2" t="s">
-        <v>269</v>
+        <v>205</v>
       </c>
       <c r="E1200" s="2" t="s">
-        <v>4660</v>
+        <v>4657</v>
       </c>
       <c r="F1200" s="2" t="s">
         <v>11</v>
@@ -41401,197 +41497,197 @@
     </row>
     <row r="1201" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1201" s="6" t="s">
-        <v>4661</v>
-      </c>
-      <c r="B1201" s="2" t="s">
-        <v>4662</v>
+        <v>4658</v>
+      </c>
+      <c r="B1201" s="4">
+        <v>80000</v>
       </c>
       <c r="C1201" s="2" t="s">
-        <v>4663</v>
+        <v>4659</v>
       </c>
       <c r="D1201" s="2" t="s">
-        <v>1304</v>
+        <v>269</v>
       </c>
       <c r="E1201" s="2" t="s">
-        <v>4664</v>
+        <v>4660</v>
       </c>
       <c r="F1201" s="2" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="G1201" s="2"/>
     </row>
     <row r="1202" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1202" s="6" t="s">
-        <v>4665</v>
+        <v>4661</v>
       </c>
       <c r="B1202" s="2" t="s">
-        <v>4666</v>
+        <v>4662</v>
       </c>
       <c r="C1202" s="2" t="s">
-        <v>4667</v>
+        <v>4663</v>
       </c>
       <c r="D1202" s="2" t="s">
-        <v>1467</v>
+        <v>1304</v>
       </c>
       <c r="E1202" s="2" t="s">
-        <v>4668</v>
+        <v>4664</v>
       </c>
       <c r="F1202" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1202" s="3">
-        <v>42017</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="G1202" s="2"/>
     </row>
     <row r="1203" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1203" s="6" t="s">
-        <v>4669</v>
+        <v>4665</v>
       </c>
       <c r="B1203" s="2" t="s">
-        <v>4670</v>
+        <v>4666</v>
       </c>
       <c r="C1203" s="2" t="s">
-        <v>3873</v>
+        <v>4667</v>
       </c>
       <c r="D1203" s="2" t="s">
-        <v>54</v>
+        <v>1467</v>
       </c>
       <c r="E1203" s="2" t="s">
-        <v>4671</v>
+        <v>4668</v>
       </c>
       <c r="F1203" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1203" s="2"/>
+      <c r="G1203" s="3">
+        <v>42017</v>
+      </c>
     </row>
     <row r="1204" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1204" s="6" t="s">
-        <v>4672</v>
+        <v>4669</v>
       </c>
       <c r="B1204" s="2" t="s">
-        <v>4673</v>
+        <v>4670</v>
       </c>
       <c r="C1204" s="2" t="s">
-        <v>4674</v>
+        <v>3873</v>
       </c>
       <c r="D1204" s="2" t="s">
-        <v>4675</v>
+        <v>54</v>
       </c>
       <c r="E1204" s="2" t="s">
-        <v>4676</v>
+        <v>4671</v>
       </c>
       <c r="F1204" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1204" s="3">
-        <v>12551</v>
-      </c>
+      <c r="G1204" s="2"/>
     </row>
     <row r="1205" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1205" s="6" t="s">
-        <v>4677</v>
+        <v>4672</v>
       </c>
       <c r="B1205" s="2" t="s">
-        <v>4678</v>
+        <v>4673</v>
       </c>
       <c r="C1205" s="2" t="s">
-        <v>4679</v>
+        <v>4674</v>
       </c>
       <c r="D1205" s="2" t="s">
-        <v>318</v>
+        <v>4675</v>
       </c>
       <c r="E1205" s="2" t="s">
-        <v>4680</v>
+        <v>4676</v>
       </c>
       <c r="F1205" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1205" s="3">
-        <v>21747</v>
+        <v>12551</v>
       </c>
     </row>
     <row r="1206" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1206" s="6" t="s">
-        <v>4681</v>
+        <v>4677</v>
       </c>
       <c r="B1206" s="2" t="s">
-        <v>4682</v>
+        <v>4678</v>
       </c>
       <c r="C1206" s="2" t="s">
         <v>4679</v>
       </c>
       <c r="D1206" s="2" t="s">
-        <v>132</v>
+        <v>318</v>
       </c>
       <c r="E1206" s="2" t="s">
-        <v>4683</v>
+        <v>4680</v>
       </c>
       <c r="F1206" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1206" s="3">
-        <v>40286</v>
+        <v>21747</v>
       </c>
     </row>
     <row r="1207" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1207" s="6" t="s">
-        <v>4684</v>
+        <v>4681</v>
       </c>
       <c r="B1207" s="2" t="s">
-        <v>4685</v>
+        <v>4682</v>
       </c>
       <c r="C1207" s="2" t="s">
-        <v>4686</v>
+        <v>4679</v>
       </c>
       <c r="D1207" s="2" t="s">
-        <v>269</v>
+        <v>132</v>
       </c>
       <c r="E1207" s="2" t="s">
-        <v>4687</v>
+        <v>4683</v>
       </c>
       <c r="F1207" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G1207" s="3">
-        <v>35163</v>
+        <v>40286</v>
       </c>
     </row>
     <row r="1208" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1208" s="6" t="s">
-        <v>4688</v>
-      </c>
-      <c r="B1208" s="2">
-        <v>201906</v>
+        <v>4684</v>
+      </c>
+      <c r="B1208" s="2" t="s">
+        <v>4685</v>
       </c>
       <c r="C1208" s="2" t="s">
         <v>4686</v>
       </c>
       <c r="D1208" s="2" t="s">
-        <v>4689</v>
+        <v>269</v>
       </c>
       <c r="E1208" s="2" t="s">
-        <v>4690</v>
+        <v>4687</v>
       </c>
       <c r="F1208" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1208" s="2"/>
+      <c r="G1208" s="3">
+        <v>35163</v>
+      </c>
     </row>
     <row r="1209" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1209" s="6" t="s">
-        <v>4691</v>
-      </c>
-      <c r="B1209" s="2" t="s">
-        <v>4692</v>
+        <v>4688</v>
+      </c>
+      <c r="B1209" s="2">
+        <v>201906</v>
       </c>
       <c r="C1209" s="2" t="s">
-        <v>4693</v>
+        <v>4686</v>
       </c>
       <c r="D1209" s="2" t="s">
-        <v>4694</v>
+        <v>4689</v>
       </c>
       <c r="E1209" s="2" t="s">
-        <v>4695</v>
+        <v>4690</v>
       </c>
       <c r="F1209" s="2" t="s">
         <v>11</v>
@@ -41600,19 +41696,19 @@
     </row>
     <row r="1210" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1210" s="6" t="s">
-        <v>4696</v>
+        <v>4691</v>
       </c>
       <c r="B1210" s="2" t="s">
-        <v>4697</v>
+        <v>4692</v>
       </c>
       <c r="C1210" s="2" t="s">
-        <v>4698</v>
+        <v>4693</v>
       </c>
       <c r="D1210" s="2" t="s">
-        <v>1462</v>
+        <v>4694</v>
       </c>
       <c r="E1210" s="2" t="s">
-        <v>4699</v>
+        <v>4695</v>
       </c>
       <c r="F1210" s="2" t="s">
         <v>11</v>
@@ -41621,19 +41717,19 @@
     </row>
     <row r="1211" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1211" s="6" t="s">
-        <v>4700</v>
+        <v>4696</v>
       </c>
       <c r="B1211" s="2" t="s">
-        <v>4701</v>
+        <v>4697</v>
       </c>
       <c r="C1211" s="2" t="s">
-        <v>4702</v>
+        <v>4698</v>
       </c>
       <c r="D1211" s="2" t="s">
-        <v>4703</v>
+        <v>1462</v>
       </c>
       <c r="E1211" s="2" t="s">
-        <v>4704</v>
+        <v>4699</v>
       </c>
       <c r="F1211" s="2" t="s">
         <v>11</v>
@@ -41642,71 +41738,75 @@
     </row>
     <row r="1212" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1212" s="6" t="s">
+        <v>4700</v>
+      </c>
+      <c r="B1212" s="2" t="s">
+        <v>4701</v>
+      </c>
+      <c r="C1212" s="2" t="s">
+        <v>4702</v>
+      </c>
+      <c r="D1212" s="2" t="s">
+        <v>4703</v>
+      </c>
+      <c r="E1212" s="2" t="s">
+        <v>4704</v>
+      </c>
+      <c r="F1212" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1212" s="2"/>
+    </row>
+    <row r="1213" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1213" s="6" t="s">
         <v>4705</v>
       </c>
-      <c r="B1212" s="2">
+      <c r="B1213" s="2">
         <v>203092</v>
       </c>
-      <c r="C1212" s="2" t="s">
+      <c r="C1213" s="2" t="s">
         <v>4706</v>
       </c>
-      <c r="D1212" s="2" t="s">
+      <c r="D1213" s="2" t="s">
         <v>4707</v>
       </c>
-      <c r="E1212" s="2" t="s">
+      <c r="E1213" s="2" t="s">
         <v>4708</v>
       </c>
-      <c r="F1212" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1212" s="2"/>
-    </row>
-    <row r="1213" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1213" s="8">
-        <v>290544</v>
-      </c>
-      <c r="C1213" t="s">
-        <v>4735</v>
-      </c>
-      <c r="D1213" t="s">
-        <v>2719</v>
-      </c>
-      <c r="E1213" t="s">
-        <v>4779</v>
-      </c>
-      <c r="F1213" t="s">
-        <v>69</v>
-      </c>
+      <c r="F1213" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1213" s="2"/>
     </row>
     <row r="1214" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1214" s="8">
-        <v>300246</v>
+        <v>290544</v>
       </c>
       <c r="C1214" t="s">
-        <v>4736</v>
+        <v>4735</v>
       </c>
       <c r="D1214" t="s">
-        <v>691</v>
+        <v>2719</v>
       </c>
       <c r="E1214" t="s">
-        <v>4780</v>
+        <v>4779</v>
       </c>
       <c r="F1214" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1215" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1215" s="8">
-        <v>288713</v>
+        <v>300246</v>
       </c>
       <c r="C1215" t="s">
-        <v>385</v>
+        <v>4736</v>
       </c>
       <c r="D1215" t="s">
-        <v>4737</v>
+        <v>691</v>
       </c>
       <c r="E1215" t="s">
-        <v>4781</v>
+        <v>4780</v>
       </c>
       <c r="F1215" t="s">
         <v>11</v>
@@ -41714,16 +41814,16 @@
     </row>
     <row r="1216" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1216" s="8">
-        <v>299498</v>
+        <v>288713</v>
       </c>
       <c r="C1216" t="s">
-        <v>4738</v>
+        <v>385</v>
       </c>
       <c r="D1216" t="s">
-        <v>757</v>
+        <v>4737</v>
       </c>
       <c r="E1216" t="s">
-        <v>4782</v>
+        <v>4781</v>
       </c>
       <c r="F1216" t="s">
         <v>11</v>
@@ -41731,16 +41831,16 @@
     </row>
     <row r="1217" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1217" s="8">
-        <v>300129</v>
+        <v>299498</v>
       </c>
       <c r="C1217" t="s">
-        <v>4739</v>
+        <v>4738</v>
       </c>
       <c r="D1217" t="s">
-        <v>4740</v>
+        <v>757</v>
       </c>
       <c r="E1217" t="s">
-        <v>4783</v>
+        <v>4782</v>
       </c>
       <c r="F1217" t="s">
         <v>11</v>
@@ -41748,101 +41848,101 @@
     </row>
     <row r="1218" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1218" s="8">
-        <v>299145</v>
+        <v>300129</v>
       </c>
       <c r="C1218" t="s">
-        <v>4741</v>
+        <v>4739</v>
       </c>
       <c r="D1218" t="s">
-        <v>4742</v>
+        <v>4740</v>
       </c>
       <c r="E1218" t="s">
-        <v>4784</v>
+        <v>4783</v>
       </c>
       <c r="F1218" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1219" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1219" s="8">
-        <v>300121</v>
+        <v>299145</v>
       </c>
       <c r="C1219" t="s">
-        <v>4743</v>
+        <v>4741</v>
       </c>
       <c r="D1219" t="s">
-        <v>4744</v>
+        <v>4742</v>
       </c>
       <c r="E1219" t="s">
-        <v>4785</v>
+        <v>4784</v>
       </c>
       <c r="F1219" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1220" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1220" s="8">
+        <v>300121</v>
+      </c>
+      <c r="C1220" t="s">
+        <v>4743</v>
+      </c>
+      <c r="D1220" t="s">
+        <v>4744</v>
+      </c>
+      <c r="E1220" t="s">
+        <v>4785</v>
+      </c>
+      <c r="F1220" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1221" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1221" s="8">
         <v>300006</v>
       </c>
-      <c r="C1220" t="s">
+      <c r="C1221" t="s">
         <v>814</v>
       </c>
-      <c r="D1220" t="s">
+      <c r="D1221" t="s">
         <v>4349</v>
       </c>
-      <c r="E1220" t="s">
+      <c r="E1221" t="s">
         <v>4786</v>
       </c>
-      <c r="F1220" t="s">
+      <c r="F1221" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="1221" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B1221" s="8" t="s">
-        <v>4732</v>
-      </c>
-      <c r="C1221" t="s">
-        <v>844</v>
-      </c>
-      <c r="D1221" t="s">
-        <v>92</v>
-      </c>
-      <c r="E1221" t="s">
-        <v>4787</v>
-      </c>
-      <c r="F1221" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="1222" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1222" s="8" t="s">
+        <v>4732</v>
+      </c>
+      <c r="C1222" t="s">
+        <v>844</v>
+      </c>
+      <c r="D1222" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1222" t="s">
+        <v>4787</v>
+      </c>
+      <c r="F1222" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1223" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1223" s="8" t="s">
         <v>4733</v>
       </c>
-      <c r="C1222" t="s">
+      <c r="C1223" t="s">
         <v>1183</v>
       </c>
-      <c r="D1222" t="s">
+      <c r="D1223" t="s">
         <v>4745</v>
       </c>
-      <c r="E1222" t="s">
+      <c r="E1223" t="s">
         <v>4788</v>
-      </c>
-      <c r="F1222" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="1223" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B1223" s="8">
-        <v>299964</v>
-      </c>
-      <c r="C1223" t="s">
-        <v>4746</v>
-      </c>
-      <c r="D1223" t="s">
-        <v>4747</v>
-      </c>
-      <c r="E1223" t="s">
-        <v>4789</v>
       </c>
       <c r="F1223" t="s">
         <v>69</v>
@@ -41850,16 +41950,16 @@
     </row>
     <row r="1224" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1224" s="8">
-        <v>295588</v>
+        <v>299964</v>
       </c>
       <c r="C1224" t="s">
-        <v>1756</v>
+        <v>4746</v>
       </c>
       <c r="D1224" t="s">
-        <v>4748</v>
+        <v>4747</v>
       </c>
       <c r="E1224" t="s">
-        <v>4790</v>
+        <v>4789</v>
       </c>
       <c r="F1224" t="s">
         <v>69</v>
@@ -41867,16 +41967,16 @@
     </row>
     <row r="1225" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1225" s="8">
-        <v>299150</v>
+        <v>295588</v>
       </c>
       <c r="C1225" t="s">
-        <v>120</v>
+        <v>1756</v>
       </c>
       <c r="D1225" t="s">
-        <v>4749</v>
+        <v>4748</v>
       </c>
       <c r="E1225" t="s">
-        <v>4791</v>
+        <v>4790</v>
       </c>
       <c r="F1225" t="s">
         <v>69</v>
@@ -41884,84 +41984,84 @@
     </row>
     <row r="1226" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1226" s="8">
-        <v>299174</v>
+        <v>299150</v>
       </c>
       <c r="C1226" t="s">
-        <v>4750</v>
+        <v>120</v>
       </c>
       <c r="D1226" t="s">
-        <v>4751</v>
+        <v>4749</v>
       </c>
       <c r="E1226" t="s">
-        <v>4792</v>
+        <v>4791</v>
       </c>
       <c r="F1226" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1227" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1227" s="8">
-        <v>295676</v>
+        <v>299174</v>
       </c>
       <c r="C1227" t="s">
-        <v>4752</v>
+        <v>4750</v>
       </c>
       <c r="D1227" t="s">
-        <v>4753</v>
+        <v>4751</v>
       </c>
       <c r="E1227" t="s">
-        <v>4793</v>
+        <v>4792</v>
       </c>
       <c r="F1227" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1228" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1228" s="8">
-        <v>300130</v>
+        <v>295676</v>
       </c>
       <c r="C1228" t="s">
-        <v>4754</v>
+        <v>4752</v>
       </c>
       <c r="D1228" t="s">
-        <v>4737</v>
+        <v>4753</v>
       </c>
       <c r="E1228" t="s">
-        <v>4794</v>
+        <v>4793</v>
       </c>
       <c r="F1228" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1229" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1229" s="8">
-        <v>298800</v>
+        <v>300130</v>
       </c>
       <c r="C1229" t="s">
-        <v>4755</v>
+        <v>4754</v>
       </c>
       <c r="D1229" t="s">
-        <v>4756</v>
+        <v>4737</v>
       </c>
       <c r="E1229" t="s">
-        <v>4795</v>
+        <v>4794</v>
       </c>
       <c r="F1229" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1230" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1230" s="8">
-        <v>296272</v>
+        <v>298800</v>
       </c>
       <c r="C1230" t="s">
-        <v>4757</v>
+        <v>4755</v>
       </c>
       <c r="D1230" t="s">
-        <v>3012</v>
+        <v>4756</v>
       </c>
       <c r="E1230" t="s">
-        <v>4796</v>
+        <v>4795</v>
       </c>
       <c r="F1230" t="s">
         <v>69</v>
@@ -41969,33 +42069,33 @@
     </row>
     <row r="1231" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1231" s="8">
-        <v>300120</v>
+        <v>296272</v>
       </c>
       <c r="C1231" t="s">
-        <v>4758</v>
+        <v>4757</v>
       </c>
       <c r="D1231" t="s">
-        <v>215</v>
+        <v>3012</v>
       </c>
       <c r="E1231" t="s">
-        <v>4797</v>
+        <v>4796</v>
       </c>
       <c r="F1231" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1232" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1232" s="8">
-        <v>300122</v>
+        <v>300120</v>
       </c>
       <c r="C1232" t="s">
-        <v>4759</v>
+        <v>4758</v>
       </c>
       <c r="D1232" t="s">
-        <v>4737</v>
+        <v>215</v>
       </c>
       <c r="E1232" t="s">
-        <v>4798</v>
+        <v>4797</v>
       </c>
       <c r="F1232" t="s">
         <v>11</v>
@@ -42003,16 +42103,16 @@
     </row>
     <row r="1233" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1233" s="8">
-        <v>300126</v>
+        <v>300122</v>
       </c>
       <c r="C1233" t="s">
-        <v>3761</v>
+        <v>4759</v>
       </c>
       <c r="D1233" t="s">
-        <v>83</v>
+        <v>4737</v>
       </c>
       <c r="E1233" t="s">
-        <v>4799</v>
+        <v>4798</v>
       </c>
       <c r="F1233" t="s">
         <v>11</v>
@@ -42020,16 +42120,16 @@
     </row>
     <row r="1234" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1234" s="8">
-        <v>298840</v>
+        <v>300126</v>
       </c>
       <c r="C1234" t="s">
-        <v>4760</v>
+        <v>3761</v>
       </c>
       <c r="D1234" t="s">
-        <v>4761</v>
+        <v>83</v>
       </c>
       <c r="E1234" t="s">
-        <v>4800</v>
+        <v>4799</v>
       </c>
       <c r="F1234" t="s">
         <v>11</v>
@@ -42037,33 +42137,33 @@
     </row>
     <row r="1235" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1235" s="8">
-        <v>157125</v>
+        <v>298840</v>
       </c>
       <c r="C1235" t="s">
-        <v>3828</v>
+        <v>4760</v>
       </c>
       <c r="D1235" t="s">
-        <v>4762</v>
+        <v>4761</v>
       </c>
       <c r="E1235" t="s">
-        <v>4801</v>
+        <v>4800</v>
       </c>
       <c r="F1235" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1236" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1236" s="8">
-        <v>297660</v>
+        <v>157125</v>
       </c>
       <c r="C1236" t="s">
-        <v>3892</v>
+        <v>3828</v>
       </c>
       <c r="D1236" t="s">
-        <v>4763</v>
+        <v>4762</v>
       </c>
       <c r="E1236" t="s">
-        <v>4802</v>
+        <v>4801</v>
       </c>
       <c r="F1236" t="s">
         <v>69</v>
@@ -42071,50 +42171,50 @@
     </row>
     <row r="1237" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1237" s="8">
-        <v>299623</v>
+        <v>297660</v>
       </c>
       <c r="C1237" t="s">
-        <v>4764</v>
+        <v>3892</v>
       </c>
       <c r="D1237" t="s">
-        <v>3287</v>
+        <v>4763</v>
       </c>
       <c r="E1237" t="s">
-        <v>4803</v>
+        <v>4802</v>
       </c>
       <c r="F1237" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="1238" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B1238" s="8" t="s">
-        <v>4734</v>
+      <c r="B1238" s="8">
+        <v>299623</v>
       </c>
       <c r="C1238" t="s">
-        <v>4765</v>
+        <v>4764</v>
       </c>
       <c r="D1238" t="s">
-        <v>4766</v>
+        <v>3287</v>
       </c>
       <c r="E1238" t="s">
-        <v>4804</v>
+        <v>4803</v>
       </c>
       <c r="F1238" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="1239" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B1239" s="8">
-        <v>298121</v>
+      <c r="B1239" s="8" t="s">
+        <v>4734</v>
       </c>
       <c r="C1239" t="s">
-        <v>4767</v>
+        <v>4765</v>
       </c>
       <c r="D1239" t="s">
-        <v>4768</v>
+        <v>4766</v>
       </c>
       <c r="E1239" t="s">
-        <v>4805</v>
+        <v>4804</v>
       </c>
       <c r="F1239" t="s">
         <v>69</v>
@@ -42122,16 +42222,16 @@
     </row>
     <row r="1240" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1240" s="8">
-        <v>286042</v>
+        <v>298121</v>
       </c>
       <c r="C1240" t="s">
-        <v>4147</v>
+        <v>4767</v>
       </c>
       <c r="D1240" t="s">
-        <v>4769</v>
+        <v>4768</v>
       </c>
       <c r="E1240" t="s">
-        <v>4806</v>
+        <v>4805</v>
       </c>
       <c r="F1240" t="s">
         <v>69</v>
@@ -42139,16 +42239,16 @@
     </row>
     <row r="1241" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1241" s="8">
-        <v>300124</v>
+        <v>286042</v>
       </c>
       <c r="C1241" t="s">
-        <v>4770</v>
+        <v>4147</v>
       </c>
       <c r="D1241" t="s">
-        <v>4771</v>
+        <v>4769</v>
       </c>
       <c r="E1241" t="s">
-        <v>4807</v>
+        <v>4806</v>
       </c>
       <c r="F1241" t="s">
         <v>69</v>
@@ -42156,50 +42256,50 @@
     </row>
     <row r="1242" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1242" s="8">
-        <v>300147</v>
+        <v>300124</v>
       </c>
       <c r="C1242" t="s">
-        <v>4772</v>
+        <v>4770</v>
       </c>
       <c r="D1242" t="s">
-        <v>4773</v>
+        <v>4771</v>
       </c>
       <c r="E1242" t="s">
-        <v>4808</v>
+        <v>4807</v>
       </c>
       <c r="F1242" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1243" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1243" s="8">
-        <v>300123</v>
+        <v>300147</v>
       </c>
       <c r="C1243" t="s">
-        <v>4774</v>
+        <v>4772</v>
       </c>
       <c r="D1243" t="s">
-        <v>4775</v>
+        <v>4773</v>
       </c>
       <c r="E1243" t="s">
-        <v>4809</v>
+        <v>4808</v>
       </c>
       <c r="F1243" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1244" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1244" s="8">
-        <v>300127</v>
+        <v>300123</v>
       </c>
       <c r="C1244" t="s">
-        <v>4776</v>
+        <v>4774</v>
       </c>
       <c r="D1244" t="s">
-        <v>957</v>
+        <v>4775</v>
       </c>
       <c r="E1244" t="s">
-        <v>4810</v>
+        <v>4809</v>
       </c>
       <c r="F1244" t="s">
         <v>69</v>
@@ -42207,40 +42307,261 @@
     </row>
     <row r="1245" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1245" s="8">
-        <v>286535</v>
+        <v>300127</v>
       </c>
       <c r="C1245" t="s">
-        <v>4777</v>
+        <v>4776</v>
       </c>
       <c r="D1245" t="s">
-        <v>92</v>
+        <v>957</v>
       </c>
       <c r="E1245" t="s">
-        <v>4811</v>
+        <v>4810</v>
       </c>
       <c r="F1245" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="1246" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1246" s="8">
+        <v>286535</v>
+      </c>
+      <c r="C1246" t="s">
+        <v>4777</v>
+      </c>
+      <c r="D1246" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1246" t="s">
+        <v>4811</v>
+      </c>
+      <c r="F1246" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1247" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1247" s="8">
         <v>235654</v>
       </c>
-      <c r="C1246" t="s">
+      <c r="C1247" t="s">
         <v>4778</v>
       </c>
-      <c r="D1246" t="s">
+      <c r="D1247" t="s">
         <v>1467</v>
       </c>
-      <c r="E1246" t="s">
+      <c r="E1247" t="s">
         <v>4812</v>
       </c>
-      <c r="F1246" t="s">
+      <c r="F1247" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1248" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1248" s="8">
+        <v>312323</v>
+      </c>
+      <c r="C1248" t="s">
+        <v>4829</v>
+      </c>
+      <c r="D1248" t="s">
+        <v>4840</v>
+      </c>
+      <c r="E1248" t="s">
+        <v>4817</v>
+      </c>
+      <c r="F1248" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1249" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1249" s="8">
+        <v>26417</v>
+      </c>
+      <c r="C1249" t="s">
+        <v>4830</v>
+      </c>
+      <c r="D1249" t="s">
+        <v>4841</v>
+      </c>
+      <c r="E1249" t="s">
+        <v>4818</v>
+      </c>
+      <c r="F1249" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1250" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1250" s="8">
+        <v>316550</v>
+      </c>
+      <c r="C1250" t="s">
+        <v>4831</v>
+      </c>
+      <c r="D1250" t="s">
+        <v>4839</v>
+      </c>
+      <c r="E1250" t="s">
+        <v>4819</v>
+      </c>
+      <c r="F1250" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1251" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1251" s="8">
+        <v>88411</v>
+      </c>
+      <c r="C1251" t="s">
+        <v>4832</v>
+      </c>
+      <c r="D1251" t="s">
+        <v>3741</v>
+      </c>
+      <c r="E1251" t="s">
+        <v>4820</v>
+      </c>
+      <c r="F1251" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1252" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1252" s="8">
+        <v>312393</v>
+      </c>
+      <c r="C1252" t="s">
+        <v>4071</v>
+      </c>
+      <c r="D1252" t="s">
+        <v>4740</v>
+      </c>
+      <c r="E1252" t="s">
+        <v>4821</v>
+      </c>
+      <c r="F1252" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1253" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1253" s="8">
+        <v>316915</v>
+      </c>
+      <c r="C1253" t="s">
+        <v>4833</v>
+      </c>
+      <c r="D1253" t="s">
+        <v>4842</v>
+      </c>
+      <c r="E1253" t="s">
+        <v>4822</v>
+      </c>
+      <c r="F1253" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1254" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1254" s="8">
+        <v>23497</v>
+      </c>
+      <c r="C1254" t="s">
+        <v>346</v>
+      </c>
+      <c r="D1254" t="s">
+        <v>4843</v>
+      </c>
+      <c r="E1254" t="s">
+        <v>4823</v>
+      </c>
+      <c r="F1254" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1255" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1255" s="8">
+        <v>248895</v>
+      </c>
+      <c r="C1255" t="s">
+        <v>4834</v>
+      </c>
+      <c r="D1255" t="s">
+        <v>4742</v>
+      </c>
+      <c r="E1255" t="s">
+        <v>4824</v>
+      </c>
+      <c r="F1255" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1256" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1256" s="8">
+        <v>11788</v>
+      </c>
+      <c r="C1256" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1256" t="s">
+        <v>1121</v>
+      </c>
+      <c r="E1256" t="s">
+        <v>4825</v>
+      </c>
+      <c r="F1256" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1257" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1257" s="8">
+        <v>315434</v>
+      </c>
+      <c r="C1257" t="s">
+        <v>4835</v>
+      </c>
+      <c r="D1257" t="s">
+        <v>4839</v>
+      </c>
+      <c r="E1257" t="s">
+        <v>4826</v>
+      </c>
+      <c r="F1257" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1258" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1258" s="8">
+        <v>316312</v>
+      </c>
+      <c r="C1258" t="s">
+        <v>4836</v>
+      </c>
+      <c r="D1258" t="s">
+        <v>540</v>
+      </c>
+      <c r="E1258" t="s">
+        <v>4827</v>
+      </c>
+      <c r="F1258" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1259" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1259" s="8">
+        <v>316547</v>
+      </c>
+      <c r="C1259" t="s">
+        <v>4837</v>
+      </c>
+      <c r="D1259" t="s">
+        <v>4838</v>
+      </c>
+      <c r="E1259" t="s">
+        <v>4828</v>
+      </c>
+      <c r="F1259" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1212" xr:uid="{19D0AC81-670F-3C42-86B4-43C7337F72FB}"/>
+  <autoFilter ref="A1:G1213" xr:uid="{19D0AC81-670F-3C42-86B4-43C7337F72FB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update mapping with names that were missed
</commit_message>
<xml_diff>
--- a/additional_data/lookup_tables/ausPH_AusPol_mapping.xlsx
+++ b/additional_data/lookup_tables/ausPH_AusPol_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindsaykatz/Documents/RA/hansard/additional_data/lookup_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6ACC0FC-3076-F248-8BED-4AAB71C9A3A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D57929-B86C-AE42-8152-FF1C7DBE2714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="840" windowWidth="27640" windowHeight="16360" xr2:uid="{3F854667-67DD-A44E-A8BA-9046689ACB2E}"/>
+    <workbookView xWindow="840" yWindow="840" windowWidth="27640" windowHeight="16360" xr2:uid="{3F854667-67DD-A44E-A8BA-9046689ACB2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7335" uniqueCount="4844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7445" uniqueCount="4901">
   <si>
     <t>uniqueID</t>
   </si>
@@ -14570,6 +14570,177 @@
   </si>
   <si>
     <t>Carol</t>
+  </si>
+  <si>
+    <t>Caldwell</t>
+  </si>
+  <si>
+    <t>Belyea</t>
+  </si>
+  <si>
+    <t>McKenzie, Zoe</t>
+  </si>
+  <si>
+    <t>Caldwell, Cameron</t>
+  </si>
+  <si>
+    <t>Kennedy, Simon</t>
+  </si>
+  <si>
+    <t>Belyea, Jodie</t>
+  </si>
+  <si>
+    <t>Ambihaipahar, Ash</t>
+  </si>
+  <si>
+    <t>Batt, David</t>
+  </si>
+  <si>
+    <t>Briskey, Jo</t>
+  </si>
+  <si>
+    <t>Campbell, Julie-Ann</t>
+  </si>
+  <si>
+    <t>Clutterham, Claire</t>
+  </si>
+  <si>
+    <t>Comer, Emma</t>
+  </si>
+  <si>
+    <t>Cook, Kara</t>
+  </si>
+  <si>
+    <t>Cook, Trish</t>
+  </si>
+  <si>
+    <t>Doyle, Mary</t>
+  </si>
+  <si>
+    <t>France, Ali</t>
+  </si>
+  <si>
+    <t>Gregg, Matt</t>
+  </si>
+  <si>
+    <t>Jarrett, Madonna</t>
+  </si>
+  <si>
+    <t>Jordan-Baird, Alice</t>
+  </si>
+  <si>
+    <t>Moncrieff, David</t>
+  </si>
+  <si>
+    <t>Ng, Gabriel</t>
+  </si>
+  <si>
+    <t>Small, Ben</t>
+  </si>
+  <si>
+    <t>Soon, Zhi</t>
+  </si>
+  <si>
+    <t>Teesdale, Jess</t>
+  </si>
+  <si>
+    <t>Urquhart, Anne</t>
+  </si>
+  <si>
+    <t>White, Rebecca</t>
+  </si>
+  <si>
+    <t>Witty, Sarah</t>
+  </si>
+  <si>
+    <t>Payne, Marise</t>
+  </si>
+  <si>
+    <t>Ambihaipahar</t>
+  </si>
+  <si>
+    <t>Ash</t>
+  </si>
+  <si>
+    <t>Jo</t>
+  </si>
+  <si>
+    <t>Julie-Ann</t>
+  </si>
+  <si>
+    <t>Claire</t>
+  </si>
+  <si>
+    <t>Kara</t>
+  </si>
+  <si>
+    <t>Trish</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>Madonna</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>Gabriel</t>
+  </si>
+  <si>
+    <t>Marise</t>
+  </si>
+  <si>
+    <t>Zhi</t>
+  </si>
+  <si>
+    <t>Rebecca</t>
+  </si>
+  <si>
+    <t>Batt</t>
+  </si>
+  <si>
+    <t>Briskey</t>
+  </si>
+  <si>
+    <t>Clutterham</t>
+  </si>
+  <si>
+    <t>Comer</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Gregg</t>
+  </si>
+  <si>
+    <t>Jarrett</t>
+  </si>
+  <si>
+    <t>Jordan-Baird</t>
+  </si>
+  <si>
+    <t>Moncrieff</t>
+  </si>
+  <si>
+    <t>Ng</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Soon</t>
+  </si>
+  <si>
+    <t>Teesdale</t>
+  </si>
+  <si>
+    <t>Witty</t>
+  </si>
+  <si>
+    <t>M56</t>
   </si>
 </sst>
 </file>
@@ -14619,7 +14790,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -14645,6 +14816,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -14960,7 +15134,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19D0AC81-670F-3C42-86B4-43C7337F72FB}">
-  <dimension ref="A1:G1259"/>
+  <dimension ref="A1:G1286"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
@@ -42560,6 +42734,465 @@
         <v>11</v>
       </c>
     </row>
+    <row r="1260" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1260" s="8">
+        <v>124514</v>
+      </c>
+      <c r="C1260" t="s">
+        <v>3175</v>
+      </c>
+      <c r="D1260" t="s">
+        <v>4745</v>
+      </c>
+      <c r="E1260" t="s">
+        <v>4846</v>
+      </c>
+      <c r="F1260" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1261" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1261" s="8">
+        <v>306489</v>
+      </c>
+      <c r="C1261" t="s">
+        <v>4844</v>
+      </c>
+      <c r="D1261" t="s">
+        <v>699</v>
+      </c>
+      <c r="E1261" t="s">
+        <v>4847</v>
+      </c>
+      <c r="F1261" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1262" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1262" s="8">
+        <v>267506</v>
+      </c>
+      <c r="C1262" t="s">
+        <v>2602</v>
+      </c>
+      <c r="D1262" t="s">
+        <v>1129</v>
+      </c>
+      <c r="E1262" t="s">
+        <v>4848</v>
+      </c>
+      <c r="F1262" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1263" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1263" s="8">
+        <v>309484</v>
+      </c>
+      <c r="C1263" t="s">
+        <v>4845</v>
+      </c>
+      <c r="D1263" t="s">
+        <v>748</v>
+      </c>
+      <c r="E1263" t="s">
+        <v>4849</v>
+      </c>
+      <c r="F1263" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1264" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1264" s="8" t="s">
+        <v>1603</v>
+      </c>
+      <c r="C1264" t="s">
+        <v>1604</v>
+      </c>
+      <c r="D1264" t="s">
+        <v>1462</v>
+      </c>
+      <c r="E1264" t="s">
+        <v>1605</v>
+      </c>
+      <c r="F1264" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1265" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1265" s="8">
+        <v>315618</v>
+      </c>
+      <c r="C1265" t="s">
+        <v>4872</v>
+      </c>
+      <c r="D1265" t="s">
+        <v>4873</v>
+      </c>
+      <c r="E1265" t="s">
+        <v>4850</v>
+      </c>
+      <c r="F1265" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1266" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1266" s="10">
+        <v>315478</v>
+      </c>
+      <c r="C1266" t="s">
+        <v>4886</v>
+      </c>
+      <c r="D1266" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1266" t="s">
+        <v>4851</v>
+      </c>
+      <c r="F1266" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1267" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1267" s="8">
+        <v>263427</v>
+      </c>
+      <c r="C1267" t="s">
+        <v>4887</v>
+      </c>
+      <c r="D1267" t="s">
+        <v>4874</v>
+      </c>
+      <c r="E1267" t="s">
+        <v>4852</v>
+      </c>
+      <c r="F1267" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1268" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1268" s="8">
+        <v>312823</v>
+      </c>
+      <c r="C1268" t="s">
+        <v>743</v>
+      </c>
+      <c r="D1268" t="s">
+        <v>4875</v>
+      </c>
+      <c r="E1268" t="s">
+        <v>4853</v>
+      </c>
+      <c r="F1268" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1269" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1269" s="8">
+        <v>316101</v>
+      </c>
+      <c r="C1269" t="s">
+        <v>4888</v>
+      </c>
+      <c r="D1269" t="s">
+        <v>4876</v>
+      </c>
+      <c r="E1269" t="s">
+        <v>4854</v>
+      </c>
+      <c r="F1269" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1270" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1270" s="8">
+        <v>316551</v>
+      </c>
+      <c r="C1270" t="s">
+        <v>4889</v>
+      </c>
+      <c r="D1270" t="s">
+        <v>2338</v>
+      </c>
+      <c r="E1270" t="s">
+        <v>4855</v>
+      </c>
+      <c r="F1270" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1271" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1271" s="8">
+        <v>316537</v>
+      </c>
+      <c r="C1271" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D1271" t="s">
+        <v>4877</v>
+      </c>
+      <c r="E1271" t="s">
+        <v>4856</v>
+      </c>
+      <c r="F1271" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1272" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1272" s="10">
+        <v>312871</v>
+      </c>
+      <c r="C1272" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D1272" t="s">
+        <v>4878</v>
+      </c>
+      <c r="E1272" t="s">
+        <v>4857</v>
+      </c>
+      <c r="F1272" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1273" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1273" s="8">
+        <v>299962</v>
+      </c>
+      <c r="C1273" t="s">
+        <v>1295</v>
+      </c>
+      <c r="D1273" t="s">
+        <v>1121</v>
+      </c>
+      <c r="E1273" t="s">
+        <v>4858</v>
+      </c>
+      <c r="F1273" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1274" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1274" s="8">
+        <v>270198</v>
+      </c>
+      <c r="C1274" t="s">
+        <v>4890</v>
+      </c>
+      <c r="D1274" t="s">
+        <v>4879</v>
+      </c>
+      <c r="E1274" t="s">
+        <v>4859</v>
+      </c>
+      <c r="F1274" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1275" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1275" s="8">
+        <v>315154</v>
+      </c>
+      <c r="C1275" t="s">
+        <v>4891</v>
+      </c>
+      <c r="D1275" t="s">
+        <v>4740</v>
+      </c>
+      <c r="E1275" t="s">
+        <v>4860</v>
+      </c>
+      <c r="F1275" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1276" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1276" s="8">
+        <v>298574</v>
+      </c>
+      <c r="C1276" t="s">
+        <v>4892</v>
+      </c>
+      <c r="D1276" t="s">
+        <v>4880</v>
+      </c>
+      <c r="E1276" t="s">
+        <v>4861</v>
+      </c>
+      <c r="F1276" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1277" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1277" s="8">
+        <v>316021</v>
+      </c>
+      <c r="C1277" t="s">
+        <v>4893</v>
+      </c>
+      <c r="D1277" t="s">
+        <v>4881</v>
+      </c>
+      <c r="E1277" t="s">
+        <v>4862</v>
+      </c>
+      <c r="F1277" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1278" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1278" s="8">
+        <v>316540</v>
+      </c>
+      <c r="C1278" t="s">
+        <v>4894</v>
+      </c>
+      <c r="D1278" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1278" t="s">
+        <v>4863</v>
+      </c>
+      <c r="F1278" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1279" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1279" s="8">
+        <v>316052</v>
+      </c>
+      <c r="C1279" t="s">
+        <v>4895</v>
+      </c>
+      <c r="D1279" t="s">
+        <v>4882</v>
+      </c>
+      <c r="E1279" t="s">
+        <v>4864</v>
+      </c>
+      <c r="F1279" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1280" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1280" s="8" t="s">
+        <v>4900</v>
+      </c>
+      <c r="C1280" t="s">
+        <v>3600</v>
+      </c>
+      <c r="D1280" t="s">
+        <v>4883</v>
+      </c>
+      <c r="E1280" t="s">
+        <v>4871</v>
+      </c>
+      <c r="F1280" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1281" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1281" s="8">
+        <v>291406</v>
+      </c>
+      <c r="C1281" t="s">
+        <v>4896</v>
+      </c>
+      <c r="D1281" t="s">
+        <v>3335</v>
+      </c>
+      <c r="E1281" t="s">
+        <v>4865</v>
+      </c>
+      <c r="F1281" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1282" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1282" s="8">
+        <v>298618</v>
+      </c>
+      <c r="C1282" t="s">
+        <v>4897</v>
+      </c>
+      <c r="D1282" t="s">
+        <v>4884</v>
+      </c>
+      <c r="E1282" t="s">
+        <v>4866</v>
+      </c>
+      <c r="F1282" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1283" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1283" s="8">
+        <v>314526</v>
+      </c>
+      <c r="C1283" t="s">
+        <v>4898</v>
+      </c>
+      <c r="D1283" t="s">
+        <v>2447</v>
+      </c>
+      <c r="E1283" t="s">
+        <v>4867</v>
+      </c>
+      <c r="F1283" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1284" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1284" s="8">
+        <v>231199</v>
+      </c>
+      <c r="C1284" t="s">
+        <v>2365</v>
+      </c>
+      <c r="D1284" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1284" t="s">
+        <v>4868</v>
+      </c>
+      <c r="F1284" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1285" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1285" s="8">
+        <v>224102</v>
+      </c>
+      <c r="C1285" t="s">
+        <v>4548</v>
+      </c>
+      <c r="D1285" t="s">
+        <v>4885</v>
+      </c>
+      <c r="E1285" t="s">
+        <v>4869</v>
+      </c>
+      <c r="F1285" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1286" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1286" s="8">
+        <v>316660</v>
+      </c>
+      <c r="C1286" t="s">
+        <v>4899</v>
+      </c>
+      <c r="D1286" t="s">
+        <v>2161</v>
+      </c>
+      <c r="E1286" t="s">
+        <v>4870</v>
+      </c>
+      <c r="F1286" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1213" xr:uid="{19D0AC81-670F-3C42-86B4-43C7337F72FB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>